<commit_message>
Schedule: Updated for day 1 Doc: Part with mockups almost done
</commit_message>
<xml_diff>
--- a/docs/PA_2023_Journal_Zeitplan_Olivier_Luethy.xlsx
+++ b/docs/PA_2023_Journal_Zeitplan_Olivier_Luethy.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="141" documentId="8_{71233B79-E4B6-4549-AD2C-3963A6ED4295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1243923-158D-40B7-AD21-D32123E026A9}"/>
+  <xr:revisionPtr revIDLastSave="200" documentId="8_{71233B79-E4B6-4549-AD2C-3963A6ED4295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0512DF55-DEB8-422D-BBF8-E43AA8D237D7}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Zeitplan" sheetId="1" r:id="rId1"/>
@@ -182,7 +182,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy;@"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -248,6 +248,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -839,7 +845,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="13"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -902,166 +908,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="4" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="4" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="13" xfId="6"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="37" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="38" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="39" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="40" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="41" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="42" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1070,6 +919,170 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="15" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="37" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="38" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="39" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="40" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="41" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="42" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Abwesenheit" xfId="5" xr:uid="{044D2A48-2EE8-4886-A796-1561124F3878}"/>
@@ -1404,170 +1417,170 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:57" x14ac:dyDescent="0.25">
-      <c r="A1" s="86" t="s">
+      <c r="A1" s="93" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="103" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="79" t="s">
+      <c r="C1" s="106" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="80"/>
-      <c r="E1" s="93" t="s">
+      <c r="D1" s="107"/>
+      <c r="E1" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="93" t="s">
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="59" t="s">
         <v>26</v>
       </c>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="95"/>
-      <c r="M1" s="93" t="s">
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="95"/>
-      <c r="Q1" s="93" t="s">
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="61"/>
+      <c r="Q1" s="59" t="s">
         <v>28</v>
       </c>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="95"/>
-      <c r="U1" s="93" t="s">
+      <c r="R1" s="60"/>
+      <c r="S1" s="60"/>
+      <c r="T1" s="61"/>
+      <c r="U1" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="95"/>
-      <c r="Y1" s="93" t="s">
+      <c r="V1" s="60"/>
+      <c r="W1" s="60"/>
+      <c r="X1" s="61"/>
+      <c r="Y1" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="95"/>
-      <c r="AC1" s="93" t="s">
+      <c r="Z1" s="60"/>
+      <c r="AA1" s="60"/>
+      <c r="AB1" s="61"/>
+      <c r="AC1" s="59" t="s">
         <v>26</v>
       </c>
-      <c r="AD1" s="94"/>
-      <c r="AE1" s="94"/>
-      <c r="AF1" s="95"/>
-      <c r="AG1" s="93" t="s">
+      <c r="AD1" s="60"/>
+      <c r="AE1" s="60"/>
+      <c r="AF1" s="61"/>
+      <c r="AG1" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="AH1" s="94"/>
-      <c r="AI1" s="94"/>
-      <c r="AJ1" s="95"/>
-      <c r="AK1" s="93" t="s">
+      <c r="AH1" s="60"/>
+      <c r="AI1" s="60"/>
+      <c r="AJ1" s="61"/>
+      <c r="AK1" s="59" t="s">
         <v>28</v>
       </c>
-      <c r="AL1" s="94"/>
-      <c r="AM1" s="94"/>
-      <c r="AN1" s="95"/>
-      <c r="AO1" s="93" t="s">
+      <c r="AL1" s="60"/>
+      <c r="AM1" s="60"/>
+      <c r="AN1" s="61"/>
+      <c r="AO1" s="59" t="s">
         <v>29</v>
       </c>
-      <c r="AP1" s="94"/>
-      <c r="AQ1" s="94"/>
-      <c r="AR1" s="95"/>
-      <c r="AS1" s="93" t="s">
+      <c r="AP1" s="60"/>
+      <c r="AQ1" s="60"/>
+      <c r="AR1" s="61"/>
+      <c r="AS1" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="AT1" s="94"/>
-      <c r="AU1" s="94"/>
-      <c r="AV1" s="95"/>
-      <c r="AW1" s="93" t="s">
+      <c r="AT1" s="60"/>
+      <c r="AU1" s="60"/>
+      <c r="AV1" s="61"/>
+      <c r="AW1" s="59" t="s">
         <v>26</v>
       </c>
-      <c r="AX1" s="94"/>
-      <c r="AY1" s="94"/>
-      <c r="AZ1" s="95"/>
+      <c r="AX1" s="60"/>
+      <c r="AY1" s="60"/>
+      <c r="AZ1" s="61"/>
     </row>
     <row r="2" spans="1:57" x14ac:dyDescent="0.25">
-      <c r="A2" s="87"/>
-      <c r="B2" s="77"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="97">
+      <c r="A2" s="94"/>
+      <c r="B2" s="104"/>
+      <c r="C2" s="108"/>
+      <c r="D2" s="109"/>
+      <c r="E2" s="62">
         <v>45001</v>
       </c>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="99"/>
-      <c r="I2" s="97">
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="62">
         <v>45002</v>
       </c>
-      <c r="J2" s="98"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="97">
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="62">
         <v>45005</v>
       </c>
-      <c r="N2" s="98"/>
-      <c r="O2" s="98"/>
-      <c r="P2" s="99"/>
-      <c r="Q2" s="97">
+      <c r="N2" s="63"/>
+      <c r="O2" s="63"/>
+      <c r="P2" s="64"/>
+      <c r="Q2" s="62">
         <v>45006</v>
       </c>
-      <c r="R2" s="98"/>
-      <c r="S2" s="98"/>
-      <c r="T2" s="99"/>
-      <c r="U2" s="97">
+      <c r="R2" s="63"/>
+      <c r="S2" s="63"/>
+      <c r="T2" s="64"/>
+      <c r="U2" s="62">
         <v>45007</v>
       </c>
-      <c r="V2" s="98"/>
-      <c r="W2" s="98"/>
-      <c r="X2" s="99"/>
-      <c r="Y2" s="97">
+      <c r="V2" s="63"/>
+      <c r="W2" s="63"/>
+      <c r="X2" s="64"/>
+      <c r="Y2" s="62">
         <v>45008</v>
       </c>
-      <c r="Z2" s="98"/>
-      <c r="AA2" s="98"/>
-      <c r="AB2" s="99"/>
-      <c r="AC2" s="97">
+      <c r="Z2" s="63"/>
+      <c r="AA2" s="63"/>
+      <c r="AB2" s="64"/>
+      <c r="AC2" s="62">
         <v>45009</v>
       </c>
-      <c r="AD2" s="98"/>
-      <c r="AE2" s="98"/>
-      <c r="AF2" s="99"/>
-      <c r="AG2" s="97">
+      <c r="AD2" s="63"/>
+      <c r="AE2" s="63"/>
+      <c r="AF2" s="64"/>
+      <c r="AG2" s="62">
         <v>45012</v>
       </c>
-      <c r="AH2" s="98"/>
-      <c r="AI2" s="98"/>
-      <c r="AJ2" s="99"/>
-      <c r="AK2" s="97">
+      <c r="AH2" s="63"/>
+      <c r="AI2" s="63"/>
+      <c r="AJ2" s="64"/>
+      <c r="AK2" s="62">
         <v>45013</v>
       </c>
-      <c r="AL2" s="98"/>
-      <c r="AM2" s="98"/>
-      <c r="AN2" s="99"/>
-      <c r="AO2" s="97">
+      <c r="AL2" s="63"/>
+      <c r="AM2" s="63"/>
+      <c r="AN2" s="64"/>
+      <c r="AO2" s="62">
         <v>45014</v>
       </c>
-      <c r="AP2" s="98"/>
-      <c r="AQ2" s="98"/>
-      <c r="AR2" s="99"/>
-      <c r="AS2" s="97">
+      <c r="AP2" s="63"/>
+      <c r="AQ2" s="63"/>
+      <c r="AR2" s="64"/>
+      <c r="AS2" s="62">
         <v>45015</v>
       </c>
-      <c r="AT2" s="98"/>
-      <c r="AU2" s="98"/>
-      <c r="AV2" s="99"/>
-      <c r="AW2" s="97">
+      <c r="AT2" s="63"/>
+      <c r="AU2" s="63"/>
+      <c r="AV2" s="64"/>
+      <c r="AW2" s="62">
         <v>45016</v>
       </c>
-      <c r="AX2" s="98"/>
-      <c r="AY2" s="98"/>
-      <c r="AZ2" s="99"/>
+      <c r="AX2" s="63"/>
+      <c r="AY2" s="63"/>
+      <c r="AZ2" s="64"/>
     </row>
     <row r="3" spans="1:57" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="88"/>
-      <c r="B3" s="78"/>
+      <c r="A3" s="95"/>
+      <c r="B3" s="105"/>
       <c r="C3" s="31" t="s">
         <v>3</v>
       </c>
@@ -1721,9 +1734,9 @@
     </row>
     <row r="4" spans="1:57" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="21"/>
-      <c r="B4" s="85"/>
-      <c r="C4" s="62"/>
-      <c r="D4" s="71"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="79"/>
+      <c r="D4" s="83"/>
       <c r="E4" s="10"/>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
@@ -1767,9 +1780,9 @@
     </row>
     <row r="5" spans="1:57" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="22"/>
-      <c r="B5" s="66"/>
-      <c r="C5" s="83"/>
-      <c r="D5" s="102"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="84"/>
       <c r="E5" s="13"/>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
@@ -1820,16 +1833,16 @@
       <c r="AZ5" s="18"/>
     </row>
     <row r="6" spans="1:57" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="96" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="91" t="s">
+      <c r="B6" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="69">
+      <c r="C6" s="82">
         <v>0.5</v>
       </c>
-      <c r="D6" s="100">
+      <c r="D6" s="80">
         <v>0.5</v>
       </c>
       <c r="E6" s="40">
@@ -1846,12 +1859,12 @@
       <c r="N6" s="8"/>
       <c r="O6" s="8"/>
       <c r="P6" s="9"/>
-      <c r="Q6" s="52" t="s">
+      <c r="Q6" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="R6" s="53"/>
-      <c r="S6" s="53"/>
-      <c r="T6" s="54"/>
+      <c r="R6" s="66"/>
+      <c r="S6" s="66"/>
+      <c r="T6" s="67"/>
       <c r="U6" s="26"/>
       <c r="V6" s="8"/>
       <c r="W6" s="8"/>
@@ -1868,12 +1881,12 @@
       <c r="AH6" s="8"/>
       <c r="AI6" s="8"/>
       <c r="AJ6" s="9"/>
-      <c r="AK6" s="52" t="s">
+      <c r="AK6" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="AL6" s="53"/>
-      <c r="AM6" s="53"/>
-      <c r="AN6" s="54"/>
+      <c r="AL6" s="66"/>
+      <c r="AM6" s="66"/>
+      <c r="AN6" s="67"/>
       <c r="AO6" s="26"/>
       <c r="AP6" s="8"/>
       <c r="AQ6" s="8"/>
@@ -1888,10 +1901,10 @@
       <c r="AZ6" s="9"/>
     </row>
     <row r="7" spans="1:57" x14ac:dyDescent="0.25">
-      <c r="A7" s="64"/>
-      <c r="B7" s="72"/>
-      <c r="C7" s="62"/>
-      <c r="D7" s="101"/>
+      <c r="A7" s="97"/>
+      <c r="B7" s="75"/>
+      <c r="C7" s="79"/>
+      <c r="D7" s="81"/>
       <c r="E7" s="45">
         <v>0.5</v>
       </c>
@@ -1906,10 +1919,10 @@
       <c r="N7" s="11"/>
       <c r="O7" s="11"/>
       <c r="P7" s="12"/>
-      <c r="Q7" s="55"/>
-      <c r="R7" s="56"/>
-      <c r="S7" s="56"/>
-      <c r="T7" s="57"/>
+      <c r="Q7" s="68"/>
+      <c r="R7" s="69"/>
+      <c r="S7" s="69"/>
+      <c r="T7" s="70"/>
       <c r="U7" s="10"/>
       <c r="V7" s="11"/>
       <c r="W7" s="11"/>
@@ -1926,10 +1939,10 @@
       <c r="AH7" s="11"/>
       <c r="AI7" s="11"/>
       <c r="AJ7" s="12"/>
-      <c r="AK7" s="55"/>
-      <c r="AL7" s="56"/>
-      <c r="AM7" s="56"/>
-      <c r="AN7" s="57"/>
+      <c r="AK7" s="68"/>
+      <c r="AL7" s="69"/>
+      <c r="AM7" s="69"/>
+      <c r="AN7" s="70"/>
       <c r="AO7" s="10"/>
       <c r="AP7" s="11"/>
       <c r="AQ7" s="11"/>
@@ -1944,14 +1957,14 @@
       <c r="AZ7" s="12"/>
     </row>
     <row r="8" spans="1:57" x14ac:dyDescent="0.25">
-      <c r="A8" s="64"/>
-      <c r="B8" s="72" t="s">
+      <c r="A8" s="97"/>
+      <c r="B8" s="75" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="96">
+      <c r="C8" s="90">
         <v>1.5</v>
       </c>
-      <c r="D8" s="96">
+      <c r="D8" s="90">
         <v>1.5</v>
       </c>
       <c r="E8" s="41">
@@ -1968,10 +1981,10 @@
       <c r="N8" s="11"/>
       <c r="O8" s="11"/>
       <c r="P8" s="12"/>
-      <c r="Q8" s="55"/>
-      <c r="R8" s="56"/>
-      <c r="S8" s="56"/>
-      <c r="T8" s="57"/>
+      <c r="Q8" s="68"/>
+      <c r="R8" s="69"/>
+      <c r="S8" s="69"/>
+      <c r="T8" s="70"/>
       <c r="U8" s="10"/>
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
@@ -1988,10 +2001,10 @@
       <c r="AH8" s="11"/>
       <c r="AI8" s="11"/>
       <c r="AJ8" s="12"/>
-      <c r="AK8" s="55"/>
-      <c r="AL8" s="56"/>
-      <c r="AM8" s="56"/>
-      <c r="AN8" s="57"/>
+      <c r="AK8" s="68"/>
+      <c r="AL8" s="69"/>
+      <c r="AM8" s="69"/>
+      <c r="AN8" s="70"/>
       <c r="AO8" s="10"/>
       <c r="AP8" s="11"/>
       <c r="AQ8" s="11"/>
@@ -2006,10 +2019,10 @@
       <c r="AZ8" s="12"/>
     </row>
     <row r="9" spans="1:57" x14ac:dyDescent="0.25">
-      <c r="A9" s="64"/>
-      <c r="B9" s="72"/>
-      <c r="C9" s="62"/>
-      <c r="D9" s="62"/>
+      <c r="A9" s="97"/>
+      <c r="B9" s="75"/>
+      <c r="C9" s="79"/>
+      <c r="D9" s="79"/>
       <c r="E9" s="45">
         <v>1.5</v>
       </c>
@@ -2024,10 +2037,10 @@
       <c r="N9" s="11"/>
       <c r="O9" s="11"/>
       <c r="P9" s="12"/>
-      <c r="Q9" s="55"/>
-      <c r="R9" s="56"/>
-      <c r="S9" s="56"/>
-      <c r="T9" s="57"/>
+      <c r="Q9" s="68"/>
+      <c r="R9" s="69"/>
+      <c r="S9" s="69"/>
+      <c r="T9" s="70"/>
       <c r="U9" s="10"/>
       <c r="V9" s="11"/>
       <c r="W9" s="11"/>
@@ -2044,10 +2057,10 @@
       <c r="AH9" s="11"/>
       <c r="AI9" s="11"/>
       <c r="AJ9" s="12"/>
-      <c r="AK9" s="55"/>
-      <c r="AL9" s="56"/>
-      <c r="AM9" s="56"/>
-      <c r="AN9" s="57"/>
+      <c r="AK9" s="68"/>
+      <c r="AL9" s="69"/>
+      <c r="AM9" s="69"/>
+      <c r="AN9" s="70"/>
       <c r="AO9" s="10"/>
       <c r="AP9" s="11"/>
       <c r="AQ9" s="11"/>
@@ -2062,15 +2075,15 @@
       <c r="AZ9" s="12"/>
     </row>
     <row r="10" spans="1:57" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="64"/>
-      <c r="B10" s="67" t="s">
+      <c r="A10" s="97"/>
+      <c r="B10" s="86" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="62">
+      <c r="C10" s="79">
         <v>1.5</v>
       </c>
-      <c r="D10" s="71">
-        <v>1.5</v>
+      <c r="D10" s="83">
+        <v>0.5</v>
       </c>
       <c r="E10" s="19"/>
       <c r="F10" s="42">
@@ -2086,10 +2099,10 @@
       <c r="N10" s="11"/>
       <c r="O10" s="11"/>
       <c r="P10" s="12"/>
-      <c r="Q10" s="55"/>
-      <c r="R10" s="56"/>
-      <c r="S10" s="56"/>
-      <c r="T10" s="57"/>
+      <c r="Q10" s="68"/>
+      <c r="R10" s="69"/>
+      <c r="S10" s="69"/>
+      <c r="T10" s="70"/>
       <c r="U10" s="19"/>
       <c r="V10" s="11"/>
       <c r="W10" s="11"/>
@@ -2106,10 +2119,10 @@
       <c r="AH10" s="11"/>
       <c r="AI10" s="11"/>
       <c r="AJ10" s="12"/>
-      <c r="AK10" s="55"/>
-      <c r="AL10" s="56"/>
-      <c r="AM10" s="56"/>
-      <c r="AN10" s="57"/>
+      <c r="AK10" s="68"/>
+      <c r="AL10" s="69"/>
+      <c r="AM10" s="69"/>
+      <c r="AN10" s="70"/>
       <c r="AO10" s="19"/>
       <c r="AP10" s="11"/>
       <c r="AQ10" s="11"/>
@@ -2128,13 +2141,13 @@
       <c r="BE10" s="2"/>
     </row>
     <row r="11" spans="1:57" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="65"/>
-      <c r="B11" s="73"/>
-      <c r="C11" s="74"/>
-      <c r="D11" s="75"/>
+      <c r="A11" s="98"/>
+      <c r="B11" s="100"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="92"/>
       <c r="E11" s="16"/>
       <c r="F11" s="46">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="G11" s="17"/>
       <c r="H11" s="18"/>
@@ -2146,10 +2159,10 @@
       <c r="N11" s="17"/>
       <c r="O11" s="17"/>
       <c r="P11" s="18"/>
-      <c r="Q11" s="55"/>
-      <c r="R11" s="56"/>
-      <c r="S11" s="56"/>
-      <c r="T11" s="57"/>
+      <c r="Q11" s="68"/>
+      <c r="R11" s="69"/>
+      <c r="S11" s="69"/>
+      <c r="T11" s="70"/>
       <c r="U11" s="16"/>
       <c r="V11" s="17"/>
       <c r="W11" s="17"/>
@@ -2166,10 +2179,10 @@
       <c r="AH11" s="17"/>
       <c r="AI11" s="17"/>
       <c r="AJ11" s="18"/>
-      <c r="AK11" s="55"/>
-      <c r="AL11" s="56"/>
-      <c r="AM11" s="56"/>
-      <c r="AN11" s="57"/>
+      <c r="AK11" s="68"/>
+      <c r="AL11" s="69"/>
+      <c r="AM11" s="69"/>
+      <c r="AN11" s="70"/>
       <c r="AO11" s="16"/>
       <c r="AP11" s="17"/>
       <c r="AQ11" s="17"/>
@@ -2188,17 +2201,17 @@
       <c r="BE11" s="3"/>
     </row>
     <row r="12" spans="1:57" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="96" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="92" t="s">
+      <c r="B12" s="101" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="69">
+      <c r="C12" s="82">
         <v>1</v>
       </c>
-      <c r="D12" s="70">
-        <v>1</v>
+      <c r="D12" s="85">
+        <v>0.5</v>
       </c>
       <c r="E12" s="26"/>
       <c r="F12" s="43">
@@ -2216,10 +2229,10 @@
       <c r="N12" s="20"/>
       <c r="O12" s="27"/>
       <c r="P12" s="9"/>
-      <c r="Q12" s="55"/>
-      <c r="R12" s="56"/>
-      <c r="S12" s="56"/>
-      <c r="T12" s="57"/>
+      <c r="Q12" s="68"/>
+      <c r="R12" s="69"/>
+      <c r="S12" s="69"/>
+      <c r="T12" s="70"/>
       <c r="U12" s="7"/>
       <c r="V12" s="20"/>
       <c r="W12" s="27"/>
@@ -2236,10 +2249,10 @@
       <c r="AH12" s="20"/>
       <c r="AI12" s="27"/>
       <c r="AJ12" s="9"/>
-      <c r="AK12" s="55"/>
-      <c r="AL12" s="56"/>
-      <c r="AM12" s="56"/>
-      <c r="AN12" s="57"/>
+      <c r="AK12" s="68"/>
+      <c r="AL12" s="69"/>
+      <c r="AM12" s="69"/>
+      <c r="AN12" s="70"/>
       <c r="AO12" s="7"/>
       <c r="AP12" s="20"/>
       <c r="AQ12" s="27"/>
@@ -2258,17 +2271,15 @@
       <c r="BE12" s="23"/>
     </row>
     <row r="13" spans="1:57" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="64"/>
-      <c r="B13" s="68"/>
-      <c r="C13" s="62"/>
-      <c r="D13" s="71"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="102"/>
+      <c r="C13" s="79"/>
+      <c r="D13" s="83"/>
       <c r="E13" s="10"/>
       <c r="F13" s="47">
         <v>0.5</v>
       </c>
-      <c r="G13" s="47">
-        <v>0.5</v>
-      </c>
+      <c r="G13" s="115"/>
       <c r="H13" s="12"/>
       <c r="I13" s="10"/>
       <c r="J13" s="11"/>
@@ -2278,10 +2289,10 @@
       <c r="N13" s="11"/>
       <c r="O13" s="11"/>
       <c r="P13" s="12"/>
-      <c r="Q13" s="55"/>
-      <c r="R13" s="56"/>
-      <c r="S13" s="56"/>
-      <c r="T13" s="57"/>
+      <c r="Q13" s="68"/>
+      <c r="R13" s="69"/>
+      <c r="S13" s="69"/>
+      <c r="T13" s="70"/>
       <c r="U13" s="10"/>
       <c r="V13" s="11"/>
       <c r="W13" s="11"/>
@@ -2298,10 +2309,10 @@
       <c r="AH13" s="11"/>
       <c r="AI13" s="11"/>
       <c r="AJ13" s="12"/>
-      <c r="AK13" s="55"/>
-      <c r="AL13" s="56"/>
-      <c r="AM13" s="56"/>
-      <c r="AN13" s="57"/>
+      <c r="AK13" s="68"/>
+      <c r="AL13" s="69"/>
+      <c r="AM13" s="69"/>
+      <c r="AN13" s="70"/>
       <c r="AO13" s="10"/>
       <c r="AP13" s="11"/>
       <c r="AQ13" s="11"/>
@@ -2320,15 +2331,15 @@
       <c r="BE13" s="25"/>
     </row>
     <row r="14" spans="1:57" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="64"/>
-      <c r="B14" s="72" t="s">
+      <c r="A14" s="97"/>
+      <c r="B14" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="62">
+      <c r="C14" s="79">
         <v>3.5</v>
       </c>
-      <c r="D14" s="71">
-        <v>3.5</v>
+      <c r="D14" s="83">
+        <v>0.5</v>
       </c>
       <c r="E14" s="10"/>
       <c r="F14" s="11"/>
@@ -2342,10 +2353,10 @@
       <c r="M14" s="10"/>
       <c r="N14" s="11"/>
       <c r="O14" s="11"/>
-      <c r="Q14" s="55"/>
-      <c r="R14" s="56"/>
-      <c r="S14" s="56"/>
-      <c r="T14" s="57"/>
+      <c r="Q14" s="68"/>
+      <c r="R14" s="69"/>
+      <c r="S14" s="69"/>
+      <c r="T14" s="70"/>
       <c r="U14" s="10"/>
       <c r="V14" s="11"/>
       <c r="W14" s="11"/>
@@ -2358,10 +2369,10 @@
       <c r="AG14" s="10"/>
       <c r="AH14" s="11"/>
       <c r="AI14" s="11"/>
-      <c r="AK14" s="55"/>
-      <c r="AL14" s="56"/>
-      <c r="AM14" s="56"/>
-      <c r="AN14" s="57"/>
+      <c r="AK14" s="68"/>
+      <c r="AL14" s="69"/>
+      <c r="AM14" s="69"/>
+      <c r="AN14" s="70"/>
       <c r="AO14" s="10"/>
       <c r="AP14" s="11"/>
       <c r="AQ14" s="11"/>
@@ -2380,16 +2391,16 @@
       <c r="BE14" s="24"/>
     </row>
     <row r="15" spans="1:57" x14ac:dyDescent="0.25">
-      <c r="A15" s="64"/>
-      <c r="B15" s="72"/>
-      <c r="C15" s="62"/>
-      <c r="D15" s="71"/>
+      <c r="A15" s="97"/>
+      <c r="B15" s="75"/>
+      <c r="C15" s="79"/>
+      <c r="D15" s="83"/>
       <c r="E15" s="10"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="47">
-        <v>1.5</v>
-      </c>
-      <c r="H15" s="48"/>
+      <c r="F15" s="112">
+        <v>0.5</v>
+      </c>
+      <c r="G15" s="113"/>
+      <c r="H15" s="114"/>
       <c r="I15" s="19"/>
       <c r="J15" s="11"/>
       <c r="K15" s="11"/>
@@ -2398,10 +2409,10 @@
       <c r="N15" s="11"/>
       <c r="O15" s="11"/>
       <c r="P15" s="12"/>
-      <c r="Q15" s="55"/>
-      <c r="R15" s="56"/>
-      <c r="S15" s="56"/>
-      <c r="T15" s="57"/>
+      <c r="Q15" s="68"/>
+      <c r="R15" s="69"/>
+      <c r="S15" s="69"/>
+      <c r="T15" s="70"/>
       <c r="U15" s="10"/>
       <c r="V15" s="11"/>
       <c r="W15" s="11"/>
@@ -2418,10 +2429,10 @@
       <c r="AH15" s="11"/>
       <c r="AI15" s="11"/>
       <c r="AJ15" s="12"/>
-      <c r="AK15" s="55"/>
-      <c r="AL15" s="56"/>
-      <c r="AM15" s="56"/>
-      <c r="AN15" s="57"/>
+      <c r="AK15" s="68"/>
+      <c r="AL15" s="69"/>
+      <c r="AM15" s="69"/>
+      <c r="AN15" s="70"/>
       <c r="AO15" s="10"/>
       <c r="AP15" s="11"/>
       <c r="AQ15" s="11"/>
@@ -2436,15 +2447,15 @@
       <c r="AZ15" s="12"/>
     </row>
     <row r="16" spans="1:57" x14ac:dyDescent="0.25">
-      <c r="A16" s="64"/>
-      <c r="B16" s="72" t="s">
+      <c r="A16" s="97"/>
+      <c r="B16" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="62">
+      <c r="C16" s="79">
         <v>1.5</v>
       </c>
-      <c r="D16" s="71">
-        <v>1.5</v>
+      <c r="D16" s="83">
+        <v>0.5</v>
       </c>
       <c r="E16" s="19"/>
       <c r="F16" s="11"/>
@@ -2460,10 +2471,10 @@
       <c r="N16" s="11"/>
       <c r="O16" s="11"/>
       <c r="P16" s="12"/>
-      <c r="Q16" s="55"/>
-      <c r="R16" s="56"/>
-      <c r="S16" s="56"/>
-      <c r="T16" s="57"/>
+      <c r="Q16" s="68"/>
+      <c r="R16" s="69"/>
+      <c r="S16" s="69"/>
+      <c r="T16" s="70"/>
       <c r="U16" s="10"/>
       <c r="V16" s="11"/>
       <c r="W16" s="11"/>
@@ -2480,10 +2491,10 @@
       <c r="AH16" s="11"/>
       <c r="AI16" s="11"/>
       <c r="AJ16" s="12"/>
-      <c r="AK16" s="55"/>
-      <c r="AL16" s="56"/>
-      <c r="AM16" s="56"/>
-      <c r="AN16" s="57"/>
+      <c r="AK16" s="68"/>
+      <c r="AL16" s="69"/>
+      <c r="AM16" s="69"/>
+      <c r="AN16" s="70"/>
       <c r="AO16" s="10"/>
       <c r="AP16" s="11"/>
       <c r="AQ16" s="11"/>
@@ -2498,17 +2509,17 @@
       <c r="AZ16" s="12"/>
     </row>
     <row r="17" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A17" s="64"/>
-      <c r="B17" s="72"/>
-      <c r="C17" s="62"/>
-      <c r="D17" s="71"/>
+      <c r="A17" s="97"/>
+      <c r="B17" s="75"/>
+      <c r="C17" s="79"/>
+      <c r="D17" s="83"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
+      <c r="F17" s="112">
+        <v>0.5</v>
+      </c>
+      <c r="G17" s="54"/>
       <c r="H17" s="12"/>
-      <c r="I17" s="45">
-        <v>1.5</v>
-      </c>
+      <c r="I17" s="117"/>
       <c r="J17" s="11"/>
       <c r="K17" s="11"/>
       <c r="L17" s="12"/>
@@ -2516,10 +2527,10 @@
       <c r="N17" s="11"/>
       <c r="O17" s="11"/>
       <c r="P17" s="12"/>
-      <c r="Q17" s="55"/>
-      <c r="R17" s="56"/>
-      <c r="S17" s="56"/>
-      <c r="T17" s="57"/>
+      <c r="Q17" s="68"/>
+      <c r="R17" s="69"/>
+      <c r="S17" s="69"/>
+      <c r="T17" s="70"/>
       <c r="U17" s="10"/>
       <c r="V17" s="11"/>
       <c r="W17" s="11"/>
@@ -2536,10 +2547,10 @@
       <c r="AH17" s="11"/>
       <c r="AI17" s="11"/>
       <c r="AJ17" s="12"/>
-      <c r="AK17" s="55"/>
-      <c r="AL17" s="56"/>
-      <c r="AM17" s="56"/>
-      <c r="AN17" s="57"/>
+      <c r="AK17" s="68"/>
+      <c r="AL17" s="69"/>
+      <c r="AM17" s="69"/>
+      <c r="AN17" s="70"/>
       <c r="AO17" s="10"/>
       <c r="AP17" s="11"/>
       <c r="AQ17" s="11"/>
@@ -2554,15 +2565,15 @@
       <c r="AZ17" s="12"/>
     </row>
     <row r="18" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A18" s="64"/>
-      <c r="B18" s="72" t="s">
+      <c r="A18" s="97"/>
+      <c r="B18" s="75" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="83">
+      <c r="C18" s="87">
         <v>1.5</v>
       </c>
-      <c r="D18" s="89">
-        <v>1.5</v>
+      <c r="D18" s="88">
+        <v>0.5</v>
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="11"/>
@@ -2580,10 +2591,10 @@
       <c r="N18" s="11"/>
       <c r="O18" s="20"/>
       <c r="P18" s="12"/>
-      <c r="Q18" s="55"/>
-      <c r="R18" s="56"/>
-      <c r="S18" s="56"/>
-      <c r="T18" s="57"/>
+      <c r="Q18" s="68"/>
+      <c r="R18" s="69"/>
+      <c r="S18" s="69"/>
+      <c r="T18" s="70"/>
       <c r="U18" s="10"/>
       <c r="V18" s="11"/>
       <c r="W18" s="11"/>
@@ -2600,10 +2611,10 @@
       <c r="AH18" s="11"/>
       <c r="AI18" s="11"/>
       <c r="AJ18" s="12"/>
-      <c r="AK18" s="55"/>
-      <c r="AL18" s="56"/>
-      <c r="AM18" s="56"/>
-      <c r="AN18" s="57"/>
+      <c r="AK18" s="68"/>
+      <c r="AL18" s="69"/>
+      <c r="AM18" s="69"/>
+      <c r="AN18" s="70"/>
       <c r="AO18" s="10"/>
       <c r="AP18" s="11"/>
       <c r="AQ18" s="11"/>
@@ -2618,30 +2629,28 @@
       <c r="AZ18" s="12"/>
     </row>
     <row r="19" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A19" s="64"/>
-      <c r="B19" s="72"/>
-      <c r="C19" s="96"/>
-      <c r="D19" s="103"/>
+      <c r="A19" s="97"/>
+      <c r="B19" s="75"/>
+      <c r="C19" s="90"/>
+      <c r="D19" s="89"/>
       <c r="E19" s="10"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
+      <c r="F19" s="112">
+        <v>0.5</v>
+      </c>
+      <c r="G19" s="54"/>
       <c r="H19" s="12"/>
-      <c r="I19" s="45">
-        <v>0.5</v>
-      </c>
-      <c r="J19" s="47">
-        <v>1</v>
-      </c>
+      <c r="I19" s="117"/>
+      <c r="J19" s="113"/>
       <c r="K19" s="11"/>
       <c r="L19" s="12"/>
       <c r="M19" s="10"/>
       <c r="N19" s="11"/>
-      <c r="O19" s="49"/>
+      <c r="O19" s="48"/>
       <c r="P19" s="15"/>
-      <c r="Q19" s="55"/>
-      <c r="R19" s="56"/>
-      <c r="S19" s="56"/>
-      <c r="T19" s="57"/>
+      <c r="Q19" s="68"/>
+      <c r="R19" s="69"/>
+      <c r="S19" s="69"/>
+      <c r="T19" s="70"/>
       <c r="U19" s="13"/>
       <c r="V19" s="14"/>
       <c r="W19" s="14"/>
@@ -2658,10 +2667,10 @@
       <c r="AH19" s="14"/>
       <c r="AI19" s="14"/>
       <c r="AJ19" s="15"/>
-      <c r="AK19" s="55"/>
-      <c r="AL19" s="56"/>
-      <c r="AM19" s="56"/>
-      <c r="AN19" s="57"/>
+      <c r="AK19" s="68"/>
+      <c r="AL19" s="69"/>
+      <c r="AM19" s="69"/>
+      <c r="AN19" s="70"/>
       <c r="AO19" s="13"/>
       <c r="AP19" s="14"/>
       <c r="AQ19" s="14"/>
@@ -2676,14 +2685,14 @@
       <c r="AZ19" s="15"/>
     </row>
     <row r="20" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="64"/>
-      <c r="B20" s="72" t="s">
+      <c r="A20" s="97"/>
+      <c r="B20" s="75" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="62">
+      <c r="C20" s="79">
         <v>1</v>
       </c>
-      <c r="D20" s="71">
+      <c r="D20" s="83">
         <v>1</v>
       </c>
       <c r="E20" s="10"/>
@@ -2698,12 +2707,12 @@
       <c r="L20" s="12"/>
       <c r="M20" s="10"/>
       <c r="N20" s="11"/>
-      <c r="O20" s="49"/>
+      <c r="O20" s="48"/>
       <c r="P20" s="15"/>
-      <c r="Q20" s="55"/>
-      <c r="R20" s="56"/>
-      <c r="S20" s="56"/>
-      <c r="T20" s="57"/>
+      <c r="Q20" s="68"/>
+      <c r="R20" s="69"/>
+      <c r="S20" s="69"/>
+      <c r="T20" s="70"/>
       <c r="U20" s="13"/>
       <c r="V20" s="14"/>
       <c r="W20" s="14"/>
@@ -2720,10 +2729,10 @@
       <c r="AH20" s="14"/>
       <c r="AI20" s="14"/>
       <c r="AJ20" s="15"/>
-      <c r="AK20" s="55"/>
-      <c r="AL20" s="56"/>
-      <c r="AM20" s="56"/>
-      <c r="AN20" s="57"/>
+      <c r="AK20" s="68"/>
+      <c r="AL20" s="69"/>
+      <c r="AM20" s="69"/>
+      <c r="AN20" s="70"/>
       <c r="AO20" s="13"/>
       <c r="AP20" s="14"/>
       <c r="AQ20" s="14"/>
@@ -2738,28 +2747,28 @@
       <c r="AZ20" s="15"/>
     </row>
     <row r="21" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="64"/>
-      <c r="B21" s="72"/>
-      <c r="C21" s="62"/>
-      <c r="D21" s="71"/>
+      <c r="A21" s="97"/>
+      <c r="B21" s="75"/>
+      <c r="C21" s="79"/>
+      <c r="D21" s="83"/>
       <c r="E21" s="10"/>
       <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
+      <c r="G21" s="112">
+        <v>0.5</v>
+      </c>
       <c r="H21" s="12"/>
       <c r="I21" s="10"/>
-      <c r="J21" s="47">
-        <v>1</v>
-      </c>
+      <c r="J21" s="113"/>
       <c r="K21" s="11"/>
       <c r="L21" s="12"/>
       <c r="M21" s="10"/>
       <c r="N21" s="11"/>
-      <c r="O21" s="49"/>
+      <c r="O21" s="48"/>
       <c r="P21" s="15"/>
-      <c r="Q21" s="55"/>
-      <c r="R21" s="56"/>
-      <c r="S21" s="56"/>
-      <c r="T21" s="57"/>
+      <c r="Q21" s="68"/>
+      <c r="R21" s="69"/>
+      <c r="S21" s="69"/>
+      <c r="T21" s="70"/>
       <c r="U21" s="13"/>
       <c r="V21" s="14"/>
       <c r="W21" s="14"/>
@@ -2776,10 +2785,10 @@
       <c r="AH21" s="14"/>
       <c r="AI21" s="14"/>
       <c r="AJ21" s="15"/>
-      <c r="AK21" s="55"/>
-      <c r="AL21" s="56"/>
-      <c r="AM21" s="56"/>
-      <c r="AN21" s="57"/>
+      <c r="AK21" s="68"/>
+      <c r="AL21" s="69"/>
+      <c r="AM21" s="69"/>
+      <c r="AN21" s="70"/>
       <c r="AO21" s="13"/>
       <c r="AP21" s="14"/>
       <c r="AQ21" s="14"/>
@@ -2794,15 +2803,15 @@
       <c r="AZ21" s="15"/>
     </row>
     <row r="22" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="64"/>
-      <c r="B22" s="72" t="s">
+      <c r="A22" s="97"/>
+      <c r="B22" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="62">
+      <c r="C22" s="79">
         <v>4</v>
       </c>
-      <c r="D22" s="71">
-        <v>7</v>
+      <c r="D22" s="83">
+        <v>3</v>
       </c>
       <c r="E22" s="13"/>
       <c r="F22" s="14"/>
@@ -2814,12 +2823,12 @@
       <c r="L22" s="44"/>
       <c r="M22" s="10"/>
       <c r="N22" s="11"/>
-      <c r="O22" s="49"/>
+      <c r="O22" s="48"/>
       <c r="P22" s="15"/>
-      <c r="Q22" s="55"/>
-      <c r="R22" s="56"/>
-      <c r="S22" s="56"/>
-      <c r="T22" s="57"/>
+      <c r="Q22" s="68"/>
+      <c r="R22" s="69"/>
+      <c r="S22" s="69"/>
+      <c r="T22" s="70"/>
       <c r="U22" s="13"/>
       <c r="V22" s="14"/>
       <c r="W22" s="14"/>
@@ -2836,10 +2845,10 @@
       <c r="AH22" s="14"/>
       <c r="AI22" s="14"/>
       <c r="AJ22" s="15"/>
-      <c r="AK22" s="55"/>
-      <c r="AL22" s="56"/>
-      <c r="AM22" s="56"/>
-      <c r="AN22" s="57"/>
+      <c r="AK22" s="68"/>
+      <c r="AL22" s="69"/>
+      <c r="AM22" s="69"/>
+      <c r="AN22" s="70"/>
       <c r="AO22" s="13"/>
       <c r="AP22" s="14"/>
       <c r="AQ22" s="14"/>
@@ -2854,28 +2863,30 @@
       <c r="AZ22" s="15"/>
     </row>
     <row r="23" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="64"/>
-      <c r="B23" s="72"/>
-      <c r="C23" s="62"/>
-      <c r="D23" s="71"/>
+      <c r="A23" s="97"/>
+      <c r="B23" s="75"/>
+      <c r="C23" s="79"/>
+      <c r="D23" s="83"/>
       <c r="E23" s="13"/>
       <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="12"/>
-      <c r="I23" s="10"/>
+      <c r="G23" s="116">
+        <v>1.5</v>
+      </c>
+      <c r="H23" s="111"/>
+      <c r="I23" s="118">
+        <v>0.5</v>
+      </c>
       <c r="J23" s="11"/>
-      <c r="K23" s="47"/>
-      <c r="L23" s="48"/>
-      <c r="M23" s="45"/>
-      <c r="N23" s="47">
-        <v>1</v>
-      </c>
-      <c r="O23" s="49"/>
+      <c r="K23" s="113"/>
+      <c r="L23" s="114"/>
+      <c r="M23" s="117"/>
+      <c r="N23" s="113"/>
+      <c r="O23" s="48"/>
       <c r="P23" s="15"/>
-      <c r="Q23" s="55"/>
-      <c r="R23" s="56"/>
-      <c r="S23" s="56"/>
-      <c r="T23" s="57"/>
+      <c r="Q23" s="68"/>
+      <c r="R23" s="69"/>
+      <c r="S23" s="69"/>
+      <c r="T23" s="70"/>
       <c r="U23" s="13"/>
       <c r="V23" s="14"/>
       <c r="W23" s="14"/>
@@ -2892,10 +2903,10 @@
       <c r="AH23" s="14"/>
       <c r="AI23" s="14"/>
       <c r="AJ23" s="15"/>
-      <c r="AK23" s="55"/>
-      <c r="AL23" s="56"/>
-      <c r="AM23" s="56"/>
-      <c r="AN23" s="57"/>
+      <c r="AK23" s="68"/>
+      <c r="AL23" s="69"/>
+      <c r="AM23" s="69"/>
+      <c r="AN23" s="70"/>
       <c r="AO23" s="13"/>
       <c r="AP23" s="14"/>
       <c r="AQ23" s="14"/>
@@ -2910,14 +2921,14 @@
       <c r="AZ23" s="15"/>
     </row>
     <row r="24" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A24" s="64"/>
-      <c r="B24" s="72" t="s">
+      <c r="A24" s="97"/>
+      <c r="B24" s="75" t="s">
         <v>6</v>
       </c>
-      <c r="C24" s="83">
+      <c r="C24" s="87">
         <v>3</v>
       </c>
-      <c r="D24" s="89">
+      <c r="D24" s="88">
         <v>0</v>
       </c>
       <c r="E24" s="13"/>
@@ -2928,16 +2939,16 @@
       <c r="J24" s="11"/>
       <c r="K24" s="11"/>
       <c r="L24" s="12"/>
-      <c r="M24" s="51"/>
-      <c r="N24" s="51">
+      <c r="M24" s="50"/>
+      <c r="N24" s="50">
         <v>1</v>
       </c>
-      <c r="O24" s="49"/>
+      <c r="O24" s="48"/>
       <c r="P24" s="15"/>
-      <c r="Q24" s="55"/>
-      <c r="R24" s="56"/>
-      <c r="S24" s="56"/>
-      <c r="T24" s="57"/>
+      <c r="Q24" s="68"/>
+      <c r="R24" s="69"/>
+      <c r="S24" s="69"/>
+      <c r="T24" s="70"/>
       <c r="U24" s="13"/>
       <c r="V24" s="14"/>
       <c r="W24" s="14"/>
@@ -2954,10 +2965,10 @@
       <c r="AH24" s="14"/>
       <c r="AI24" s="14"/>
       <c r="AJ24" s="15"/>
-      <c r="AK24" s="55"/>
-      <c r="AL24" s="56"/>
-      <c r="AM24" s="56"/>
-      <c r="AN24" s="57"/>
+      <c r="AK24" s="68"/>
+      <c r="AL24" s="69"/>
+      <c r="AM24" s="69"/>
+      <c r="AN24" s="70"/>
       <c r="AO24" s="13"/>
       <c r="AP24" s="14"/>
       <c r="AQ24" s="14"/>
@@ -2972,10 +2983,10 @@
       <c r="AZ24" s="15"/>
     </row>
     <row r="25" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="65"/>
-      <c r="B25" s="72"/>
-      <c r="C25" s="84"/>
-      <c r="D25" s="90"/>
+      <c r="A25" s="98"/>
+      <c r="B25" s="75"/>
+      <c r="C25" s="110"/>
+      <c r="D25" s="99"/>
       <c r="E25" s="16"/>
       <c r="F25" s="17"/>
       <c r="G25" s="17"/>
@@ -2986,12 +2997,12 @@
       <c r="L25" s="12"/>
       <c r="M25" s="19"/>
       <c r="N25" s="11"/>
-      <c r="O25" s="50"/>
+      <c r="O25" s="49"/>
       <c r="P25" s="18"/>
-      <c r="Q25" s="55"/>
-      <c r="R25" s="56"/>
-      <c r="S25" s="56"/>
-      <c r="T25" s="57"/>
+      <c r="Q25" s="68"/>
+      <c r="R25" s="69"/>
+      <c r="S25" s="69"/>
+      <c r="T25" s="70"/>
       <c r="U25" s="16"/>
       <c r="V25" s="17"/>
       <c r="W25" s="17"/>
@@ -3008,10 +3019,10 @@
       <c r="AH25" s="17"/>
       <c r="AI25" s="17"/>
       <c r="AJ25" s="18"/>
-      <c r="AK25" s="55"/>
-      <c r="AL25" s="56"/>
-      <c r="AM25" s="56"/>
-      <c r="AN25" s="57"/>
+      <c r="AK25" s="68"/>
+      <c r="AL25" s="69"/>
+      <c r="AM25" s="69"/>
+      <c r="AN25" s="70"/>
       <c r="AO25" s="16"/>
       <c r="AP25" s="17"/>
       <c r="AQ25" s="17"/>
@@ -3026,16 +3037,16 @@
       <c r="AZ25" s="18"/>
     </row>
     <row r="26" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A26" s="63" t="s">
+      <c r="A26" s="96" t="s">
         <v>10</v>
       </c>
-      <c r="B26" s="91" t="s">
+      <c r="B26" s="74" t="s">
         <v>11</v>
       </c>
-      <c r="C26" s="69">
+      <c r="C26" s="82">
         <v>1</v>
       </c>
-      <c r="D26" s="70">
+      <c r="D26" s="85">
         <v>1</v>
       </c>
       <c r="E26" s="7"/>
@@ -3052,10 +3063,10 @@
       </c>
       <c r="O26" s="8"/>
       <c r="P26" s="9"/>
-      <c r="Q26" s="55"/>
-      <c r="R26" s="56"/>
-      <c r="S26" s="56"/>
-      <c r="T26" s="57"/>
+      <c r="Q26" s="68"/>
+      <c r="R26" s="69"/>
+      <c r="S26" s="69"/>
+      <c r="T26" s="70"/>
       <c r="U26" s="7"/>
       <c r="V26" s="8"/>
       <c r="W26" s="8"/>
@@ -3072,10 +3083,10 @@
       <c r="AH26" s="8"/>
       <c r="AI26" s="8"/>
       <c r="AJ26" s="9"/>
-      <c r="AK26" s="55"/>
-      <c r="AL26" s="56"/>
-      <c r="AM26" s="56"/>
-      <c r="AN26" s="57"/>
+      <c r="AK26" s="68"/>
+      <c r="AL26" s="69"/>
+      <c r="AM26" s="69"/>
+      <c r="AN26" s="70"/>
       <c r="AO26" s="7"/>
       <c r="AP26" s="8"/>
       <c r="AQ26" s="8"/>
@@ -3090,10 +3101,10 @@
       <c r="AZ26" s="9"/>
     </row>
     <row r="27" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="64"/>
-      <c r="B27" s="73"/>
-      <c r="C27" s="74"/>
-      <c r="D27" s="75"/>
+      <c r="A27" s="97"/>
+      <c r="B27" s="100"/>
+      <c r="C27" s="91"/>
+      <c r="D27" s="92"/>
       <c r="E27" s="16"/>
       <c r="F27" s="17"/>
       <c r="G27" s="17"/>
@@ -3108,10 +3119,10 @@
       </c>
       <c r="O27" s="17"/>
       <c r="P27" s="17"/>
-      <c r="Q27" s="55"/>
-      <c r="R27" s="56"/>
-      <c r="S27" s="56"/>
-      <c r="T27" s="57"/>
+      <c r="Q27" s="68"/>
+      <c r="R27" s="69"/>
+      <c r="S27" s="69"/>
+      <c r="T27" s="70"/>
       <c r="U27" s="16"/>
       <c r="V27" s="17"/>
       <c r="W27" s="17"/>
@@ -3128,10 +3139,10 @@
       <c r="AH27" s="17"/>
       <c r="AI27" s="17"/>
       <c r="AJ27" s="18"/>
-      <c r="AK27" s="55"/>
-      <c r="AL27" s="56"/>
-      <c r="AM27" s="56"/>
-      <c r="AN27" s="57"/>
+      <c r="AK27" s="68"/>
+      <c r="AL27" s="69"/>
+      <c r="AM27" s="69"/>
+      <c r="AN27" s="70"/>
       <c r="AO27" s="16"/>
       <c r="AP27" s="17"/>
       <c r="AQ27" s="17"/>
@@ -3146,16 +3157,16 @@
       <c r="AZ27" s="18"/>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A28" s="63" t="s">
+      <c r="A28" s="96" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="91" t="s">
+      <c r="B28" s="74" t="s">
         <v>35</v>
       </c>
-      <c r="C28" s="69">
+      <c r="C28" s="82">
         <v>12</v>
       </c>
-      <c r="D28" s="70">
+      <c r="D28" s="85">
         <v>0</v>
       </c>
       <c r="E28" s="7"/>
@@ -3168,16 +3179,16 @@
       <c r="L28" s="9"/>
       <c r="M28" s="10"/>
       <c r="N28" s="11"/>
-      <c r="O28" s="104"/>
-      <c r="P28" s="105"/>
-      <c r="Q28" s="55"/>
-      <c r="R28" s="56"/>
-      <c r="S28" s="56"/>
-      <c r="T28" s="57"/>
-      <c r="U28" s="106"/>
-      <c r="V28" s="104"/>
-      <c r="W28" s="104"/>
-      <c r="X28" s="105"/>
+      <c r="O28" s="51"/>
+      <c r="P28" s="52"/>
+      <c r="Q28" s="68"/>
+      <c r="R28" s="69"/>
+      <c r="S28" s="69"/>
+      <c r="T28" s="70"/>
+      <c r="U28" s="53"/>
+      <c r="V28" s="51"/>
+      <c r="W28" s="51"/>
+      <c r="X28" s="52"/>
       <c r="Y28" s="7"/>
       <c r="Z28" s="8"/>
       <c r="AA28" s="8"/>
@@ -3190,10 +3201,10 @@
       <c r="AH28" s="8"/>
       <c r="AI28" s="8"/>
       <c r="AJ28" s="9"/>
-      <c r="AK28" s="55"/>
-      <c r="AL28" s="56"/>
-      <c r="AM28" s="56"/>
-      <c r="AN28" s="57"/>
+      <c r="AK28" s="68"/>
+      <c r="AL28" s="69"/>
+      <c r="AM28" s="69"/>
+      <c r="AN28" s="70"/>
       <c r="AO28" s="7"/>
       <c r="AP28" s="8"/>
       <c r="AQ28" s="8"/>
@@ -3208,10 +3219,10 @@
       <c r="AZ28" s="9"/>
     </row>
     <row r="29" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A29" s="64"/>
-      <c r="B29" s="72"/>
-      <c r="C29" s="62"/>
-      <c r="D29" s="71"/>
+      <c r="A29" s="97"/>
+      <c r="B29" s="75"/>
+      <c r="C29" s="79"/>
+      <c r="D29" s="83"/>
       <c r="E29" s="10"/>
       <c r="F29" s="11"/>
       <c r="G29" s="11"/>
@@ -3224,10 +3235,10 @@
       <c r="N29" s="11"/>
       <c r="O29" s="11"/>
       <c r="P29" s="36"/>
-      <c r="Q29" s="55"/>
-      <c r="R29" s="56"/>
-      <c r="S29" s="56"/>
-      <c r="T29" s="57"/>
+      <c r="Q29" s="68"/>
+      <c r="R29" s="69"/>
+      <c r="S29" s="69"/>
+      <c r="T29" s="70"/>
       <c r="U29" s="10"/>
       <c r="V29" s="11"/>
       <c r="W29" s="11"/>
@@ -3244,10 +3255,10 @@
       <c r="AH29" s="11"/>
       <c r="AI29" s="11"/>
       <c r="AJ29" s="12"/>
-      <c r="AK29" s="55"/>
-      <c r="AL29" s="56"/>
-      <c r="AM29" s="56"/>
-      <c r="AN29" s="57"/>
+      <c r="AK29" s="68"/>
+      <c r="AL29" s="69"/>
+      <c r="AM29" s="69"/>
+      <c r="AN29" s="70"/>
       <c r="AO29" s="10"/>
       <c r="AP29" s="11"/>
       <c r="AQ29" s="11"/>
@@ -3262,14 +3273,14 @@
       <c r="AZ29" s="12"/>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A30" s="64"/>
-      <c r="B30" s="66" t="s">
+      <c r="A30" s="97"/>
+      <c r="B30" s="77" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="62">
+      <c r="C30" s="79">
         <v>8</v>
       </c>
-      <c r="D30" s="71">
+      <c r="D30" s="83">
         <v>0</v>
       </c>
       <c r="E30" s="10"/>
@@ -3284,18 +3295,18 @@
       <c r="N30" s="11"/>
       <c r="O30" s="11"/>
       <c r="P30" s="36"/>
-      <c r="Q30" s="55"/>
-      <c r="R30" s="56"/>
-      <c r="S30" s="56"/>
-      <c r="T30" s="57"/>
+      <c r="Q30" s="68"/>
+      <c r="R30" s="69"/>
+      <c r="S30" s="69"/>
+      <c r="T30" s="70"/>
       <c r="U30" s="10"/>
       <c r="V30" s="11"/>
       <c r="W30" s="11"/>
       <c r="X30" s="36"/>
-      <c r="Y30" s="106"/>
-      <c r="Z30" s="104"/>
-      <c r="AA30" s="104"/>
-      <c r="AB30" s="105"/>
+      <c r="Y30" s="53"/>
+      <c r="Z30" s="51"/>
+      <c r="AA30" s="51"/>
+      <c r="AB30" s="52"/>
       <c r="AC30" s="10"/>
       <c r="AD30" s="11"/>
       <c r="AE30" s="11"/>
@@ -3304,10 +3315,10 @@
       <c r="AH30" s="11"/>
       <c r="AI30" s="11"/>
       <c r="AJ30" s="12"/>
-      <c r="AK30" s="55"/>
-      <c r="AL30" s="56"/>
-      <c r="AM30" s="56"/>
-      <c r="AN30" s="57"/>
+      <c r="AK30" s="68"/>
+      <c r="AL30" s="69"/>
+      <c r="AM30" s="69"/>
+      <c r="AN30" s="70"/>
       <c r="AO30" s="10"/>
       <c r="AP30" s="11"/>
       <c r="AQ30" s="11"/>
@@ -3322,10 +3333,10 @@
       <c r="AZ30" s="12"/>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A31" s="64"/>
-      <c r="B31" s="67"/>
-      <c r="C31" s="62"/>
-      <c r="D31" s="71"/>
+      <c r="A31" s="97"/>
+      <c r="B31" s="86"/>
+      <c r="C31" s="79"/>
+      <c r="D31" s="83"/>
       <c r="E31" s="10"/>
       <c r="F31" s="11"/>
       <c r="G31" s="11"/>
@@ -3338,10 +3349,10 @@
       <c r="N31" s="11"/>
       <c r="O31" s="11"/>
       <c r="P31" s="36"/>
-      <c r="Q31" s="55"/>
-      <c r="R31" s="56"/>
-      <c r="S31" s="56"/>
-      <c r="T31" s="57"/>
+      <c r="Q31" s="68"/>
+      <c r="R31" s="69"/>
+      <c r="S31" s="69"/>
+      <c r="T31" s="70"/>
       <c r="U31" s="10"/>
       <c r="V31" s="11"/>
       <c r="W31" s="11"/>
@@ -3358,10 +3369,10 @@
       <c r="AH31" s="11"/>
       <c r="AI31" s="11"/>
       <c r="AJ31" s="12"/>
-      <c r="AK31" s="55"/>
-      <c r="AL31" s="56"/>
-      <c r="AM31" s="56"/>
-      <c r="AN31" s="57"/>
+      <c r="AK31" s="68"/>
+      <c r="AL31" s="69"/>
+      <c r="AM31" s="69"/>
+      <c r="AN31" s="70"/>
       <c r="AO31" s="10"/>
       <c r="AP31" s="11"/>
       <c r="AQ31" s="11"/>
@@ -3376,14 +3387,14 @@
       <c r="AZ31" s="12"/>
     </row>
     <row r="32" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A32" s="64"/>
-      <c r="B32" s="66" t="s">
+      <c r="A32" s="97"/>
+      <c r="B32" s="77" t="s">
         <v>40</v>
       </c>
-      <c r="C32" s="61">
+      <c r="C32" s="78">
         <v>0.5</v>
       </c>
-      <c r="D32" s="71">
+      <c r="D32" s="83">
         <v>0</v>
       </c>
       <c r="E32" s="10"/>
@@ -3398,10 +3409,10 @@
       <c r="N32" s="11"/>
       <c r="O32" s="11"/>
       <c r="P32" s="36"/>
-      <c r="Q32" s="55"/>
-      <c r="R32" s="56"/>
-      <c r="S32" s="56"/>
-      <c r="T32" s="57"/>
+      <c r="Q32" s="68"/>
+      <c r="R32" s="69"/>
+      <c r="S32" s="69"/>
+      <c r="T32" s="70"/>
       <c r="U32" s="10"/>
       <c r="V32" s="11"/>
       <c r="W32" s="11"/>
@@ -3410,7 +3421,7 @@
       <c r="Z32" s="11"/>
       <c r="AA32" s="11"/>
       <c r="AB32" s="36"/>
-      <c r="AC32" s="106">
+      <c r="AC32" s="53">
         <v>0.5</v>
       </c>
       <c r="AD32" s="11"/>
@@ -3420,10 +3431,10 @@
       <c r="AH32" s="11"/>
       <c r="AI32" s="11"/>
       <c r="AJ32" s="12"/>
-      <c r="AK32" s="55"/>
-      <c r="AL32" s="56"/>
-      <c r="AM32" s="56"/>
-      <c r="AN32" s="57"/>
+      <c r="AK32" s="68"/>
+      <c r="AL32" s="69"/>
+      <c r="AM32" s="69"/>
+      <c r="AN32" s="70"/>
       <c r="AO32" s="10"/>
       <c r="AP32" s="11"/>
       <c r="AQ32" s="11"/>
@@ -3438,10 +3449,10 @@
       <c r="AZ32" s="12"/>
     </row>
     <row r="33" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A33" s="64"/>
-      <c r="B33" s="67"/>
-      <c r="C33" s="61"/>
-      <c r="D33" s="71"/>
+      <c r="A33" s="97"/>
+      <c r="B33" s="86"/>
+      <c r="C33" s="78"/>
+      <c r="D33" s="83"/>
       <c r="E33" s="10"/>
       <c r="F33" s="11"/>
       <c r="G33" s="11"/>
@@ -3454,10 +3465,10 @@
       <c r="N33" s="11"/>
       <c r="O33" s="11"/>
       <c r="P33" s="36"/>
-      <c r="Q33" s="55"/>
-      <c r="R33" s="56"/>
-      <c r="S33" s="56"/>
-      <c r="T33" s="57"/>
+      <c r="Q33" s="68"/>
+      <c r="R33" s="69"/>
+      <c r="S33" s="69"/>
+      <c r="T33" s="70"/>
       <c r="U33" s="10"/>
       <c r="V33" s="11"/>
       <c r="W33" s="11"/>
@@ -3474,10 +3485,10 @@
       <c r="AH33" s="11"/>
       <c r="AI33" s="11"/>
       <c r="AJ33" s="12"/>
-      <c r="AK33" s="55"/>
-      <c r="AL33" s="56"/>
-      <c r="AM33" s="56"/>
-      <c r="AN33" s="57"/>
+      <c r="AK33" s="68"/>
+      <c r="AL33" s="69"/>
+      <c r="AM33" s="69"/>
+      <c r="AN33" s="70"/>
       <c r="AO33" s="10"/>
       <c r="AP33" s="11"/>
       <c r="AQ33" s="11"/>
@@ -3492,14 +3503,14 @@
       <c r="AZ33" s="12"/>
     </row>
     <row r="34" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A34" s="64"/>
-      <c r="B34" s="66" t="s">
+      <c r="A34" s="97"/>
+      <c r="B34" s="77" t="s">
         <v>41</v>
       </c>
-      <c r="C34" s="61">
+      <c r="C34" s="78">
         <v>0.5</v>
       </c>
-      <c r="D34" s="71">
+      <c r="D34" s="83">
         <v>0</v>
       </c>
       <c r="E34" s="10"/>
@@ -3514,10 +3525,10 @@
       <c r="N34" s="11"/>
       <c r="O34" s="11"/>
       <c r="P34" s="36"/>
-      <c r="Q34" s="55"/>
-      <c r="R34" s="56"/>
-      <c r="S34" s="56"/>
-      <c r="T34" s="57"/>
+      <c r="Q34" s="68"/>
+      <c r="R34" s="69"/>
+      <c r="S34" s="69"/>
+      <c r="T34" s="70"/>
       <c r="U34" s="10"/>
       <c r="V34" s="11"/>
       <c r="W34" s="11"/>
@@ -3526,7 +3537,7 @@
       <c r="Z34" s="11"/>
       <c r="AA34" s="11"/>
       <c r="AB34" s="36"/>
-      <c r="AC34" s="106">
+      <c r="AC34" s="53">
         <v>0.5</v>
       </c>
       <c r="AD34" s="11"/>
@@ -3536,10 +3547,10 @@
       <c r="AH34" s="11"/>
       <c r="AI34" s="11"/>
       <c r="AJ34" s="12"/>
-      <c r="AK34" s="55"/>
-      <c r="AL34" s="56"/>
-      <c r="AM34" s="56"/>
-      <c r="AN34" s="57"/>
+      <c r="AK34" s="68"/>
+      <c r="AL34" s="69"/>
+      <c r="AM34" s="69"/>
+      <c r="AN34" s="70"/>
       <c r="AO34" s="10"/>
       <c r="AP34" s="11"/>
       <c r="AQ34" s="11"/>
@@ -3554,10 +3565,10 @@
       <c r="AZ34" s="12"/>
     </row>
     <row r="35" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A35" s="64"/>
-      <c r="B35" s="67"/>
-      <c r="C35" s="61"/>
-      <c r="D35" s="71"/>
+      <c r="A35" s="97"/>
+      <c r="B35" s="86"/>
+      <c r="C35" s="78"/>
+      <c r="D35" s="83"/>
       <c r="E35" s="10"/>
       <c r="F35" s="11"/>
       <c r="G35" s="11"/>
@@ -3570,10 +3581,10 @@
       <c r="N35" s="11"/>
       <c r="O35" s="11"/>
       <c r="P35" s="36"/>
-      <c r="Q35" s="55"/>
-      <c r="R35" s="56"/>
-      <c r="S35" s="56"/>
-      <c r="T35" s="57"/>
+      <c r="Q35" s="68"/>
+      <c r="R35" s="69"/>
+      <c r="S35" s="69"/>
+      <c r="T35" s="70"/>
       <c r="U35" s="10"/>
       <c r="V35" s="11"/>
       <c r="W35" s="11"/>
@@ -3590,10 +3601,10 @@
       <c r="AH35" s="11"/>
       <c r="AI35" s="11"/>
       <c r="AJ35" s="12"/>
-      <c r="AK35" s="55"/>
-      <c r="AL35" s="56"/>
-      <c r="AM35" s="56"/>
-      <c r="AN35" s="57"/>
+      <c r="AK35" s="68"/>
+      <c r="AL35" s="69"/>
+      <c r="AM35" s="69"/>
+      <c r="AN35" s="70"/>
       <c r="AO35" s="10"/>
       <c r="AP35" s="11"/>
       <c r="AQ35" s="11"/>
@@ -3608,14 +3619,14 @@
       <c r="AZ35" s="12"/>
     </row>
     <row r="36" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A36" s="64"/>
-      <c r="B36" s="66" t="s">
+      <c r="A36" s="97"/>
+      <c r="B36" s="77" t="s">
         <v>36</v>
       </c>
-      <c r="C36" s="61">
+      <c r="C36" s="78">
         <v>7</v>
       </c>
-      <c r="D36" s="61">
+      <c r="D36" s="78">
         <v>0</v>
       </c>
       <c r="E36" s="10"/>
@@ -3630,10 +3641,10 @@
       <c r="N36" s="11"/>
       <c r="O36" s="11"/>
       <c r="P36" s="36"/>
-      <c r="Q36" s="55"/>
-      <c r="R36" s="56"/>
-      <c r="S36" s="56"/>
-      <c r="T36" s="57"/>
+      <c r="Q36" s="68"/>
+      <c r="R36" s="69"/>
+      <c r="S36" s="69"/>
+      <c r="T36" s="70"/>
       <c r="U36" s="10"/>
       <c r="V36" s="11"/>
       <c r="W36" s="11"/>
@@ -3642,20 +3653,20 @@
       <c r="Z36" s="11"/>
       <c r="AA36" s="11"/>
       <c r="AB36" s="36"/>
-      <c r="AC36" s="106">
+      <c r="AC36" s="53">
         <v>1</v>
       </c>
-      <c r="AD36" s="104"/>
-      <c r="AE36" s="104"/>
-      <c r="AF36" s="105"/>
+      <c r="AD36" s="51"/>
+      <c r="AE36" s="51"/>
+      <c r="AF36" s="52"/>
       <c r="AG36" s="10"/>
       <c r="AH36" s="11"/>
       <c r="AI36" s="11"/>
       <c r="AJ36" s="12"/>
-      <c r="AK36" s="55"/>
-      <c r="AL36" s="56"/>
-      <c r="AM36" s="56"/>
-      <c r="AN36" s="57"/>
+      <c r="AK36" s="68"/>
+      <c r="AL36" s="69"/>
+      <c r="AM36" s="69"/>
+      <c r="AN36" s="70"/>
       <c r="AO36" s="10"/>
       <c r="AP36" s="11"/>
       <c r="AQ36" s="11"/>
@@ -3670,10 +3681,10 @@
       <c r="AZ36" s="12"/>
     </row>
     <row r="37" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A37" s="64"/>
-      <c r="B37" s="67"/>
-      <c r="C37" s="61"/>
-      <c r="D37" s="61"/>
+      <c r="A37" s="97"/>
+      <c r="B37" s="86"/>
+      <c r="C37" s="78"/>
+      <c r="D37" s="78"/>
       <c r="E37" s="10"/>
       <c r="F37" s="11"/>
       <c r="G37" s="11"/>
@@ -3686,10 +3697,10 @@
       <c r="N37" s="11"/>
       <c r="O37" s="11"/>
       <c r="P37" s="36"/>
-      <c r="Q37" s="55"/>
-      <c r="R37" s="56"/>
-      <c r="S37" s="56"/>
-      <c r="T37" s="57"/>
+      <c r="Q37" s="68"/>
+      <c r="R37" s="69"/>
+      <c r="S37" s="69"/>
+      <c r="T37" s="70"/>
       <c r="U37" s="10"/>
       <c r="V37" s="11"/>
       <c r="W37" s="11"/>
@@ -3706,10 +3717,10 @@
       <c r="AH37" s="11"/>
       <c r="AI37" s="11"/>
       <c r="AJ37" s="12"/>
-      <c r="AK37" s="55"/>
-      <c r="AL37" s="56"/>
-      <c r="AM37" s="56"/>
-      <c r="AN37" s="57"/>
+      <c r="AK37" s="68"/>
+      <c r="AL37" s="69"/>
+      <c r="AM37" s="69"/>
+      <c r="AN37" s="70"/>
       <c r="AO37" s="10"/>
       <c r="AP37" s="11"/>
       <c r="AQ37" s="11"/>
@@ -3724,14 +3735,14 @@
       <c r="AZ37" s="12"/>
     </row>
     <row r="38" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A38" s="64"/>
-      <c r="B38" s="66" t="s">
+      <c r="A38" s="97"/>
+      <c r="B38" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="C38" s="61">
+      <c r="C38" s="78">
         <v>0.5</v>
       </c>
-      <c r="D38" s="71">
+      <c r="D38" s="83">
         <v>0</v>
       </c>
       <c r="E38" s="10"/>
@@ -3746,10 +3757,10 @@
       <c r="N38" s="11"/>
       <c r="O38" s="11"/>
       <c r="P38" s="36"/>
-      <c r="Q38" s="55"/>
-      <c r="R38" s="56"/>
-      <c r="S38" s="56"/>
-      <c r="T38" s="57"/>
+      <c r="Q38" s="68"/>
+      <c r="R38" s="69"/>
+      <c r="S38" s="69"/>
+      <c r="T38" s="70"/>
       <c r="U38" s="10"/>
       <c r="V38" s="11"/>
       <c r="W38" s="11"/>
@@ -3762,16 +3773,16 @@
       <c r="AD38" s="11"/>
       <c r="AE38" s="11"/>
       <c r="AF38" s="12"/>
-      <c r="AG38" s="106">
+      <c r="AG38" s="53">
         <v>0.5</v>
       </c>
       <c r="AH38" s="11"/>
       <c r="AI38" s="11"/>
       <c r="AJ38" s="12"/>
-      <c r="AK38" s="55"/>
-      <c r="AL38" s="56"/>
-      <c r="AM38" s="56"/>
-      <c r="AN38" s="57"/>
+      <c r="AK38" s="68"/>
+      <c r="AL38" s="69"/>
+      <c r="AM38" s="69"/>
+      <c r="AN38" s="70"/>
       <c r="AO38" s="10"/>
       <c r="AP38" s="11"/>
       <c r="AQ38" s="11"/>
@@ -3786,10 +3797,10 @@
       <c r="AZ38" s="12"/>
     </row>
     <row r="39" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A39" s="64"/>
-      <c r="B39" s="67"/>
-      <c r="C39" s="62"/>
-      <c r="D39" s="71"/>
+      <c r="A39" s="97"/>
+      <c r="B39" s="86"/>
+      <c r="C39" s="79"/>
+      <c r="D39" s="83"/>
       <c r="E39" s="10"/>
       <c r="F39" s="11"/>
       <c r="G39" s="11"/>
@@ -3802,10 +3813,10 @@
       <c r="N39" s="11"/>
       <c r="O39" s="11"/>
       <c r="P39" s="36"/>
-      <c r="Q39" s="55"/>
-      <c r="R39" s="56"/>
-      <c r="S39" s="56"/>
-      <c r="T39" s="57"/>
+      <c r="Q39" s="68"/>
+      <c r="R39" s="69"/>
+      <c r="S39" s="69"/>
+      <c r="T39" s="70"/>
       <c r="U39" s="10"/>
       <c r="V39" s="11"/>
       <c r="W39" s="11"/>
@@ -3822,10 +3833,10 @@
       <c r="AH39" s="11"/>
       <c r="AI39" s="11"/>
       <c r="AJ39" s="12"/>
-      <c r="AK39" s="55"/>
-      <c r="AL39" s="56"/>
-      <c r="AM39" s="56"/>
-      <c r="AN39" s="57"/>
+      <c r="AK39" s="68"/>
+      <c r="AL39" s="69"/>
+      <c r="AM39" s="69"/>
+      <c r="AN39" s="70"/>
       <c r="AO39" s="10"/>
       <c r="AP39" s="11"/>
       <c r="AQ39" s="11"/>
@@ -3840,14 +3851,14 @@
       <c r="AZ39" s="12"/>
     </row>
     <row r="40" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A40" s="64"/>
-      <c r="B40" s="66" t="s">
+      <c r="A40" s="97"/>
+      <c r="B40" s="77" t="s">
         <v>43</v>
       </c>
-      <c r="C40" s="61">
+      <c r="C40" s="78">
         <v>0.5</v>
       </c>
-      <c r="D40" s="71">
+      <c r="D40" s="83">
         <v>0</v>
       </c>
       <c r="E40" s="10"/>
@@ -3862,10 +3873,10 @@
       <c r="N40" s="11"/>
       <c r="O40" s="11"/>
       <c r="P40" s="36"/>
-      <c r="Q40" s="55"/>
-      <c r="R40" s="56"/>
-      <c r="S40" s="56"/>
-      <c r="T40" s="57"/>
+      <c r="Q40" s="68"/>
+      <c r="R40" s="69"/>
+      <c r="S40" s="69"/>
+      <c r="T40" s="70"/>
       <c r="U40" s="10"/>
       <c r="V40" s="11"/>
       <c r="W40" s="11"/>
@@ -3878,16 +3889,16 @@
       <c r="AD40" s="11"/>
       <c r="AE40" s="11"/>
       <c r="AF40" s="36"/>
-      <c r="AG40" s="106">
+      <c r="AG40" s="53">
         <v>0.5</v>
       </c>
       <c r="AH40" s="11"/>
       <c r="AI40" s="11"/>
       <c r="AJ40" s="36"/>
-      <c r="AK40" s="55"/>
-      <c r="AL40" s="56"/>
-      <c r="AM40" s="56"/>
-      <c r="AN40" s="57"/>
+      <c r="AK40" s="68"/>
+      <c r="AL40" s="69"/>
+      <c r="AM40" s="69"/>
+      <c r="AN40" s="70"/>
       <c r="AO40" s="10"/>
       <c r="AP40" s="11"/>
       <c r="AQ40" s="11"/>
@@ -3902,10 +3913,10 @@
       <c r="AZ40" s="12"/>
     </row>
     <row r="41" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A41" s="64"/>
-      <c r="B41" s="67"/>
-      <c r="C41" s="62"/>
-      <c r="D41" s="71"/>
+      <c r="A41" s="97"/>
+      <c r="B41" s="86"/>
+      <c r="C41" s="79"/>
+      <c r="D41" s="83"/>
       <c r="E41" s="10"/>
       <c r="F41" s="11"/>
       <c r="G41" s="11"/>
@@ -3918,10 +3929,10 @@
       <c r="N41" s="11"/>
       <c r="O41" s="11"/>
       <c r="P41" s="12"/>
-      <c r="Q41" s="55"/>
-      <c r="R41" s="56"/>
-      <c r="S41" s="56"/>
-      <c r="T41" s="57"/>
+      <c r="Q41" s="68"/>
+      <c r="R41" s="69"/>
+      <c r="S41" s="69"/>
+      <c r="T41" s="70"/>
       <c r="U41" s="10"/>
       <c r="V41" s="11"/>
       <c r="W41" s="11"/>
@@ -3938,10 +3949,10 @@
       <c r="AH41" s="11"/>
       <c r="AI41" s="11"/>
       <c r="AJ41" s="36"/>
-      <c r="AK41" s="55"/>
-      <c r="AL41" s="56"/>
-      <c r="AM41" s="56"/>
-      <c r="AN41" s="57"/>
+      <c r="AK41" s="68"/>
+      <c r="AL41" s="69"/>
+      <c r="AM41" s="69"/>
+      <c r="AN41" s="70"/>
       <c r="AO41" s="10"/>
       <c r="AP41" s="11"/>
       <c r="AQ41" s="11"/>
@@ -3956,14 +3967,14 @@
       <c r="AZ41" s="12"/>
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A42" s="64"/>
-      <c r="B42" s="66" t="s">
+      <c r="A42" s="97"/>
+      <c r="B42" s="77" t="s">
         <v>39</v>
       </c>
-      <c r="C42" s="61">
+      <c r="C42" s="78">
         <v>0.5</v>
       </c>
-      <c r="D42" s="61">
+      <c r="D42" s="78">
         <v>0</v>
       </c>
       <c r="E42" s="10"/>
@@ -3978,10 +3989,10 @@
       <c r="N42" s="11"/>
       <c r="O42" s="11"/>
       <c r="P42" s="12"/>
-      <c r="Q42" s="55"/>
-      <c r="R42" s="56"/>
-      <c r="S42" s="56"/>
-      <c r="T42" s="57"/>
+      <c r="Q42" s="68"/>
+      <c r="R42" s="69"/>
+      <c r="S42" s="69"/>
+      <c r="T42" s="70"/>
       <c r="U42" s="10"/>
       <c r="V42" s="11"/>
       <c r="W42" s="11"/>
@@ -3994,16 +4005,16 @@
       <c r="AD42" s="11"/>
       <c r="AE42" s="11"/>
       <c r="AF42" s="36"/>
-      <c r="AG42" s="106">
+      <c r="AG42" s="53">
         <v>0.5</v>
       </c>
       <c r="AH42" s="11"/>
       <c r="AI42" s="11"/>
       <c r="AJ42" s="36"/>
-      <c r="AK42" s="55"/>
-      <c r="AL42" s="56"/>
-      <c r="AM42" s="56"/>
-      <c r="AN42" s="57"/>
+      <c r="AK42" s="68"/>
+      <c r="AL42" s="69"/>
+      <c r="AM42" s="69"/>
+      <c r="AN42" s="70"/>
       <c r="AO42" s="10"/>
       <c r="AP42" s="11"/>
       <c r="AQ42" s="11"/>
@@ -4018,10 +4029,10 @@
       <c r="AZ42" s="12"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A43" s="64"/>
-      <c r="B43" s="67"/>
-      <c r="C43" s="62"/>
-      <c r="D43" s="61"/>
+      <c r="A43" s="97"/>
+      <c r="B43" s="86"/>
+      <c r="C43" s="79"/>
+      <c r="D43" s="78"/>
       <c r="E43" s="10"/>
       <c r="F43" s="11"/>
       <c r="G43" s="11"/>
@@ -4034,10 +4045,10 @@
       <c r="N43" s="33"/>
       <c r="O43" s="33"/>
       <c r="P43" s="36"/>
-      <c r="Q43" s="55"/>
-      <c r="R43" s="56"/>
-      <c r="S43" s="56"/>
-      <c r="T43" s="57"/>
+      <c r="Q43" s="68"/>
+      <c r="R43" s="69"/>
+      <c r="S43" s="69"/>
+      <c r="T43" s="70"/>
       <c r="U43" s="10"/>
       <c r="V43" s="11"/>
       <c r="W43" s="11"/>
@@ -4054,10 +4065,10 @@
       <c r="AH43" s="11"/>
       <c r="AI43" s="11"/>
       <c r="AJ43" s="36"/>
-      <c r="AK43" s="55"/>
-      <c r="AL43" s="56"/>
-      <c r="AM43" s="56"/>
-      <c r="AN43" s="57"/>
+      <c r="AK43" s="68"/>
+      <c r="AL43" s="69"/>
+      <c r="AM43" s="69"/>
+      <c r="AN43" s="70"/>
       <c r="AO43" s="10"/>
       <c r="AP43" s="11"/>
       <c r="AQ43" s="11"/>
@@ -4072,14 +4083,14 @@
       <c r="AZ43" s="12"/>
     </row>
     <row r="44" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A44" s="64"/>
-      <c r="B44" s="66" t="s">
+      <c r="A44" s="97"/>
+      <c r="B44" s="77" t="s">
         <v>38</v>
       </c>
-      <c r="C44" s="61">
+      <c r="C44" s="78">
         <v>2.5</v>
       </c>
-      <c r="D44" s="61">
+      <c r="D44" s="78">
         <v>0</v>
       </c>
       <c r="E44" s="10"/>
@@ -4094,10 +4105,10 @@
       <c r="N44" s="33"/>
       <c r="O44" s="33"/>
       <c r="P44" s="36"/>
-      <c r="Q44" s="55"/>
-      <c r="R44" s="56"/>
-      <c r="S44" s="56"/>
-      <c r="T44" s="57"/>
+      <c r="Q44" s="68"/>
+      <c r="R44" s="69"/>
+      <c r="S44" s="69"/>
+      <c r="T44" s="70"/>
       <c r="U44" s="10"/>
       <c r="V44" s="11"/>
       <c r="W44" s="11"/>
@@ -4110,16 +4121,16 @@
       <c r="AD44" s="11"/>
       <c r="AE44" s="11"/>
       <c r="AF44" s="36"/>
-      <c r="AG44" s="106">
+      <c r="AG44" s="53">
         <v>0.5</v>
       </c>
-      <c r="AH44" s="107"/>
+      <c r="AH44" s="54"/>
       <c r="AI44" s="11"/>
       <c r="AJ44" s="36"/>
-      <c r="AK44" s="55"/>
-      <c r="AL44" s="56"/>
-      <c r="AM44" s="56"/>
-      <c r="AN44" s="57"/>
+      <c r="AK44" s="68"/>
+      <c r="AL44" s="69"/>
+      <c r="AM44" s="69"/>
+      <c r="AN44" s="70"/>
       <c r="AO44" s="10"/>
       <c r="AP44" s="11"/>
       <c r="AQ44" s="11"/>
@@ -4134,10 +4145,10 @@
       <c r="AZ44" s="12"/>
     </row>
     <row r="45" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A45" s="64"/>
-      <c r="B45" s="67"/>
-      <c r="C45" s="62"/>
-      <c r="D45" s="62"/>
+      <c r="A45" s="97"/>
+      <c r="B45" s="86"/>
+      <c r="C45" s="79"/>
+      <c r="D45" s="79"/>
       <c r="E45" s="10"/>
       <c r="F45" s="11"/>
       <c r="G45" s="11"/>
@@ -4150,10 +4161,10 @@
       <c r="N45" s="33"/>
       <c r="O45" s="33"/>
       <c r="P45" s="36"/>
-      <c r="Q45" s="55"/>
-      <c r="R45" s="56"/>
-      <c r="S45" s="56"/>
-      <c r="T45" s="57"/>
+      <c r="Q45" s="68"/>
+      <c r="R45" s="69"/>
+      <c r="S45" s="69"/>
+      <c r="T45" s="70"/>
       <c r="U45" s="10"/>
       <c r="V45" s="11"/>
       <c r="W45" s="11"/>
@@ -4170,10 +4181,10 @@
       <c r="AH45" s="11"/>
       <c r="AI45" s="11"/>
       <c r="AJ45" s="36"/>
-      <c r="AK45" s="55"/>
-      <c r="AL45" s="56"/>
-      <c r="AM45" s="56"/>
-      <c r="AN45" s="57"/>
+      <c r="AK45" s="68"/>
+      <c r="AL45" s="69"/>
+      <c r="AM45" s="69"/>
+      <c r="AN45" s="70"/>
       <c r="AO45" s="10"/>
       <c r="AP45" s="11"/>
       <c r="AQ45" s="11"/>
@@ -4188,14 +4199,14 @@
       <c r="AZ45" s="12"/>
     </row>
     <row r="46" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A46" s="64"/>
-      <c r="B46" s="66" t="s">
+      <c r="A46" s="97"/>
+      <c r="B46" s="77" t="s">
         <v>45</v>
       </c>
-      <c r="C46" s="61">
+      <c r="C46" s="78">
         <v>6</v>
       </c>
-      <c r="D46" s="61">
+      <c r="D46" s="78">
         <v>0</v>
       </c>
       <c r="E46" s="10"/>
@@ -4210,10 +4221,10 @@
       <c r="N46" s="33"/>
       <c r="O46" s="33"/>
       <c r="P46" s="36"/>
-      <c r="Q46" s="55"/>
-      <c r="R46" s="56"/>
-      <c r="S46" s="56"/>
-      <c r="T46" s="57"/>
+      <c r="Q46" s="68"/>
+      <c r="R46" s="69"/>
+      <c r="S46" s="69"/>
+      <c r="T46" s="70"/>
       <c r="U46" s="10"/>
       <c r="V46" s="11"/>
       <c r="W46" s="11"/>
@@ -4226,16 +4237,16 @@
       <c r="AD46" s="11"/>
       <c r="AE46" s="11"/>
       <c r="AF46" s="36"/>
-      <c r="AG46" s="110"/>
-      <c r="AH46" s="104"/>
-      <c r="AI46" s="104"/>
-      <c r="AJ46" s="105"/>
-      <c r="AK46" s="55"/>
-      <c r="AL46" s="56"/>
-      <c r="AM46" s="56"/>
-      <c r="AN46" s="57"/>
-      <c r="AO46" s="106"/>
-      <c r="AP46" s="104"/>
+      <c r="AG46" s="57"/>
+      <c r="AH46" s="51"/>
+      <c r="AI46" s="51"/>
+      <c r="AJ46" s="52"/>
+      <c r="AK46" s="68"/>
+      <c r="AL46" s="69"/>
+      <c r="AM46" s="69"/>
+      <c r="AN46" s="70"/>
+      <c r="AO46" s="53"/>
+      <c r="AP46" s="51"/>
       <c r="AQ46" s="11"/>
       <c r="AR46" s="12"/>
       <c r="AS46" s="10"/>
@@ -4248,10 +4259,10 @@
       <c r="AZ46" s="12"/>
     </row>
     <row r="47" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A47" s="64"/>
-      <c r="B47" s="67"/>
-      <c r="C47" s="62"/>
-      <c r="D47" s="62"/>
+      <c r="A47" s="97"/>
+      <c r="B47" s="86"/>
+      <c r="C47" s="79"/>
+      <c r="D47" s="79"/>
       <c r="E47" s="10"/>
       <c r="F47" s="11"/>
       <c r="G47" s="11"/>
@@ -4264,10 +4275,10 @@
       <c r="N47" s="11"/>
       <c r="O47" s="33"/>
       <c r="P47" s="36"/>
-      <c r="Q47" s="55"/>
-      <c r="R47" s="56"/>
-      <c r="S47" s="56"/>
-      <c r="T47" s="57"/>
+      <c r="Q47" s="68"/>
+      <c r="R47" s="69"/>
+      <c r="S47" s="69"/>
+      <c r="T47" s="70"/>
       <c r="U47" s="10"/>
       <c r="V47" s="11"/>
       <c r="W47" s="11"/>
@@ -4284,10 +4295,10 @@
       <c r="AH47" s="11"/>
       <c r="AI47" s="11"/>
       <c r="AJ47" s="36"/>
-      <c r="AK47" s="55"/>
-      <c r="AL47" s="56"/>
-      <c r="AM47" s="56"/>
-      <c r="AN47" s="57"/>
+      <c r="AK47" s="68"/>
+      <c r="AL47" s="69"/>
+      <c r="AM47" s="69"/>
+      <c r="AN47" s="70"/>
       <c r="AO47" s="10"/>
       <c r="AP47" s="11"/>
       <c r="AQ47" s="11"/>
@@ -4302,14 +4313,14 @@
       <c r="AZ47" s="12"/>
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A48" s="64"/>
-      <c r="B48" s="66" t="s">
+      <c r="A48" s="97"/>
+      <c r="B48" s="77" t="s">
         <v>44</v>
       </c>
-      <c r="C48" s="61">
+      <c r="C48" s="78">
         <v>4</v>
       </c>
-      <c r="D48" s="61">
+      <c r="D48" s="78">
         <v>0</v>
       </c>
       <c r="E48" s="10"/>
@@ -4324,10 +4335,10 @@
       <c r="N48" s="11"/>
       <c r="O48" s="33"/>
       <c r="P48" s="36"/>
-      <c r="Q48" s="55"/>
-      <c r="R48" s="56"/>
-      <c r="S48" s="56"/>
-      <c r="T48" s="57"/>
+      <c r="Q48" s="68"/>
+      <c r="R48" s="69"/>
+      <c r="S48" s="69"/>
+      <c r="T48" s="70"/>
       <c r="U48" s="10"/>
       <c r="V48" s="11"/>
       <c r="W48" s="11"/>
@@ -4344,14 +4355,14 @@
       <c r="AH48" s="11"/>
       <c r="AI48" s="11"/>
       <c r="AJ48" s="36"/>
-      <c r="AK48" s="55"/>
-      <c r="AL48" s="56"/>
-      <c r="AM48" s="56"/>
-      <c r="AN48" s="57"/>
+      <c r="AK48" s="68"/>
+      <c r="AL48" s="69"/>
+      <c r="AM48" s="69"/>
+      <c r="AN48" s="70"/>
       <c r="AO48" s="10"/>
       <c r="AP48" s="11"/>
-      <c r="AQ48" s="104"/>
-      <c r="AR48" s="105"/>
+      <c r="AQ48" s="51"/>
+      <c r="AR48" s="52"/>
       <c r="AS48" s="10"/>
       <c r="AT48" s="11"/>
       <c r="AU48" s="11"/>
@@ -4362,10 +4373,10 @@
       <c r="AZ48" s="36"/>
     </row>
     <row r="49" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A49" s="64"/>
-      <c r="B49" s="67"/>
-      <c r="C49" s="62"/>
-      <c r="D49" s="62"/>
+      <c r="A49" s="97"/>
+      <c r="B49" s="86"/>
+      <c r="C49" s="79"/>
+      <c r="D49" s="79"/>
       <c r="E49" s="10"/>
       <c r="F49" s="11"/>
       <c r="G49" s="11"/>
@@ -4378,10 +4389,10 @@
       <c r="N49" s="11"/>
       <c r="O49" s="33"/>
       <c r="P49" s="36"/>
-      <c r="Q49" s="55"/>
-      <c r="R49" s="56"/>
-      <c r="S49" s="56"/>
-      <c r="T49" s="57"/>
+      <c r="Q49" s="68"/>
+      <c r="R49" s="69"/>
+      <c r="S49" s="69"/>
+      <c r="T49" s="70"/>
       <c r="U49" s="10"/>
       <c r="V49" s="11"/>
       <c r="W49" s="11"/>
@@ -4398,10 +4409,10 @@
       <c r="AH49" s="11"/>
       <c r="AI49" s="11"/>
       <c r="AJ49" s="36"/>
-      <c r="AK49" s="55"/>
-      <c r="AL49" s="56"/>
-      <c r="AM49" s="56"/>
-      <c r="AN49" s="57"/>
+      <c r="AK49" s="68"/>
+      <c r="AL49" s="69"/>
+      <c r="AM49" s="69"/>
+      <c r="AN49" s="70"/>
       <c r="AO49" s="10"/>
       <c r="AP49" s="11"/>
       <c r="AQ49" s="11"/>
@@ -4416,14 +4427,14 @@
       <c r="AZ49" s="36"/>
     </row>
     <row r="50" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A50" s="64"/>
-      <c r="B50" s="85" t="s">
+      <c r="A50" s="97"/>
+      <c r="B50" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="C50" s="62">
+      <c r="C50" s="79">
         <v>1</v>
       </c>
-      <c r="D50" s="71">
+      <c r="D50" s="83">
         <v>0</v>
       </c>
       <c r="E50" s="10"/>
@@ -4438,10 +4449,10 @@
       <c r="N50" s="11"/>
       <c r="O50" s="11"/>
       <c r="P50" s="36"/>
-      <c r="Q50" s="55"/>
-      <c r="R50" s="56"/>
-      <c r="S50" s="56"/>
-      <c r="T50" s="57"/>
+      <c r="Q50" s="68"/>
+      <c r="R50" s="69"/>
+      <c r="S50" s="69"/>
+      <c r="T50" s="70"/>
       <c r="U50" s="10"/>
       <c r="V50" s="11"/>
       <c r="W50" s="11"/>
@@ -4458,18 +4469,18 @@
       <c r="AH50" s="11"/>
       <c r="AI50" s="11"/>
       <c r="AJ50" s="36"/>
-      <c r="AK50" s="55"/>
-      <c r="AL50" s="56"/>
-      <c r="AM50" s="56"/>
-      <c r="AN50" s="57"/>
+      <c r="AK50" s="68"/>
+      <c r="AL50" s="69"/>
+      <c r="AM50" s="69"/>
+      <c r="AN50" s="70"/>
       <c r="AO50" s="10"/>
       <c r="AP50" s="11"/>
       <c r="AQ50" s="11"/>
       <c r="AR50" s="36"/>
-      <c r="AS50" s="106">
+      <c r="AS50" s="53">
         <v>1</v>
       </c>
-      <c r="AT50" s="107"/>
+      <c r="AT50" s="54"/>
       <c r="AU50" s="11"/>
       <c r="AV50" s="36"/>
       <c r="AW50" s="10"/>
@@ -4478,10 +4489,10 @@
       <c r="AZ50" s="36"/>
     </row>
     <row r="51" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A51" s="64"/>
-      <c r="B51" s="85"/>
-      <c r="C51" s="62"/>
-      <c r="D51" s="71"/>
+      <c r="A51" s="97"/>
+      <c r="B51" s="76"/>
+      <c r="C51" s="79"/>
+      <c r="D51" s="83"/>
       <c r="E51" s="35"/>
       <c r="F51" s="33"/>
       <c r="G51" s="33"/>
@@ -4494,10 +4505,10 @@
       <c r="N51" s="33"/>
       <c r="O51" s="33"/>
       <c r="P51" s="36"/>
-      <c r="Q51" s="55"/>
-      <c r="R51" s="56"/>
-      <c r="S51" s="56"/>
-      <c r="T51" s="57"/>
+      <c r="Q51" s="68"/>
+      <c r="R51" s="69"/>
+      <c r="S51" s="69"/>
+      <c r="T51" s="70"/>
       <c r="U51" s="35"/>
       <c r="V51" s="33"/>
       <c r="W51" s="33"/>
@@ -4514,10 +4525,10 @@
       <c r="AH51" s="11"/>
       <c r="AI51" s="11"/>
       <c r="AJ51" s="36"/>
-      <c r="AK51" s="55"/>
-      <c r="AL51" s="56"/>
-      <c r="AM51" s="56"/>
-      <c r="AN51" s="57"/>
+      <c r="AK51" s="68"/>
+      <c r="AL51" s="69"/>
+      <c r="AM51" s="69"/>
+      <c r="AN51" s="70"/>
       <c r="AO51" s="10"/>
       <c r="AP51" s="11"/>
       <c r="AQ51" s="11"/>
@@ -4532,14 +4543,14 @@
       <c r="AZ51" s="36"/>
     </row>
     <row r="52" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A52" s="64"/>
-      <c r="B52" s="72" t="s">
+      <c r="A52" s="97"/>
+      <c r="B52" s="75" t="s">
         <v>6</v>
       </c>
-      <c r="C52" s="62">
+      <c r="C52" s="79">
         <v>0</v>
       </c>
-      <c r="D52" s="71">
+      <c r="D52" s="83">
         <v>0</v>
       </c>
       <c r="E52" s="10"/>
@@ -4554,10 +4565,10 @@
       <c r="N52" s="11"/>
       <c r="O52" s="11"/>
       <c r="P52" s="12"/>
-      <c r="Q52" s="55"/>
-      <c r="R52" s="56"/>
-      <c r="S52" s="56"/>
-      <c r="T52" s="57"/>
+      <c r="Q52" s="68"/>
+      <c r="R52" s="69"/>
+      <c r="S52" s="69"/>
+      <c r="T52" s="70"/>
       <c r="U52" s="10"/>
       <c r="V52" s="11"/>
       <c r="W52" s="11"/>
@@ -4574,10 +4585,10 @@
       <c r="AH52" s="11"/>
       <c r="AI52" s="11"/>
       <c r="AJ52" s="36"/>
-      <c r="AK52" s="55"/>
-      <c r="AL52" s="56"/>
-      <c r="AM52" s="56"/>
-      <c r="AN52" s="57"/>
+      <c r="AK52" s="68"/>
+      <c r="AL52" s="69"/>
+      <c r="AM52" s="69"/>
+      <c r="AN52" s="70"/>
       <c r="AO52" s="10"/>
       <c r="AP52" s="11"/>
       <c r="AQ52" s="11"/>
@@ -4592,10 +4603,10 @@
       <c r="AZ52" s="12"/>
     </row>
     <row r="53" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="64"/>
-      <c r="B53" s="72"/>
-      <c r="C53" s="62"/>
-      <c r="D53" s="71"/>
+      <c r="A53" s="97"/>
+      <c r="B53" s="75"/>
+      <c r="C53" s="79"/>
+      <c r="D53" s="83"/>
       <c r="E53" s="10"/>
       <c r="F53" s="11"/>
       <c r="G53" s="11"/>
@@ -4608,10 +4619,10 @@
       <c r="N53" s="11"/>
       <c r="O53" s="11"/>
       <c r="P53" s="12"/>
-      <c r="Q53" s="55"/>
-      <c r="R53" s="56"/>
-      <c r="S53" s="56"/>
-      <c r="T53" s="57"/>
+      <c r="Q53" s="68"/>
+      <c r="R53" s="69"/>
+      <c r="S53" s="69"/>
+      <c r="T53" s="70"/>
       <c r="U53" s="10"/>
       <c r="V53" s="11"/>
       <c r="W53" s="11"/>
@@ -4628,10 +4639,10 @@
       <c r="AH53" s="33"/>
       <c r="AI53" s="33"/>
       <c r="AJ53" s="36"/>
-      <c r="AK53" s="55"/>
-      <c r="AL53" s="56"/>
-      <c r="AM53" s="56"/>
-      <c r="AN53" s="57"/>
+      <c r="AK53" s="68"/>
+      <c r="AL53" s="69"/>
+      <c r="AM53" s="69"/>
+      <c r="AN53" s="70"/>
       <c r="AO53" s="10"/>
       <c r="AP53" s="33"/>
       <c r="AQ53" s="33"/>
@@ -4646,16 +4657,16 @@
       <c r="AZ53" s="12"/>
     </row>
     <row r="54" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A54" s="63" t="s">
+      <c r="A54" s="96" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="91" t="s">
+      <c r="B54" s="74" t="s">
         <v>19</v>
       </c>
-      <c r="C54" s="69">
+      <c r="C54" s="82">
         <v>7.5</v>
       </c>
-      <c r="D54" s="70">
+      <c r="D54" s="85">
         <v>0</v>
       </c>
       <c r="E54" s="7"/>
@@ -4670,10 +4681,10 @@
       <c r="N54" s="8"/>
       <c r="O54" s="8"/>
       <c r="P54" s="9"/>
-      <c r="Q54" s="55"/>
-      <c r="R54" s="56"/>
-      <c r="S54" s="56"/>
-      <c r="T54" s="57"/>
+      <c r="Q54" s="68"/>
+      <c r="R54" s="69"/>
+      <c r="S54" s="69"/>
+      <c r="T54" s="70"/>
       <c r="U54" s="37"/>
       <c r="V54" s="8"/>
       <c r="W54" s="8"/>
@@ -4690,30 +4701,30 @@
       <c r="AH54" s="8"/>
       <c r="AI54" s="8"/>
       <c r="AJ54" s="9"/>
-      <c r="AK54" s="55"/>
-      <c r="AL54" s="56"/>
-      <c r="AM54" s="56"/>
-      <c r="AN54" s="57"/>
+      <c r="AK54" s="68"/>
+      <c r="AL54" s="69"/>
+      <c r="AM54" s="69"/>
+      <c r="AN54" s="70"/>
       <c r="AO54" s="7"/>
       <c r="AP54" s="8"/>
       <c r="AQ54" s="8"/>
       <c r="AR54" s="9"/>
-      <c r="AS54" s="111">
+      <c r="AS54" s="58">
         <v>1</v>
       </c>
-      <c r="AT54" s="108"/>
-      <c r="AU54" s="108"/>
-      <c r="AV54" s="109"/>
+      <c r="AT54" s="55"/>
+      <c r="AU54" s="55"/>
+      <c r="AV54" s="56"/>
       <c r="AW54" s="7"/>
       <c r="AX54" s="8"/>
       <c r="AY54" s="8"/>
       <c r="AZ54" s="9"/>
     </row>
     <row r="55" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A55" s="64"/>
-      <c r="B55" s="72"/>
-      <c r="C55" s="62"/>
-      <c r="D55" s="71"/>
+      <c r="A55" s="97"/>
+      <c r="B55" s="75"/>
+      <c r="C55" s="79"/>
+      <c r="D55" s="83"/>
       <c r="E55" s="10"/>
       <c r="F55" s="11"/>
       <c r="G55" s="11"/>
@@ -4726,10 +4737,10 @@
       <c r="N55" s="11"/>
       <c r="O55" s="11"/>
       <c r="P55" s="12"/>
-      <c r="Q55" s="55"/>
-      <c r="R55" s="56"/>
-      <c r="S55" s="56"/>
-      <c r="T55" s="57"/>
+      <c r="Q55" s="68"/>
+      <c r="R55" s="69"/>
+      <c r="S55" s="69"/>
+      <c r="T55" s="70"/>
       <c r="U55" s="35"/>
       <c r="V55" s="33"/>
       <c r="W55" s="33"/>
@@ -4746,10 +4757,10 @@
       <c r="AH55" s="11"/>
       <c r="AI55" s="11"/>
       <c r="AJ55" s="36"/>
-      <c r="AK55" s="55"/>
-      <c r="AL55" s="56"/>
-      <c r="AM55" s="56"/>
-      <c r="AN55" s="57"/>
+      <c r="AK55" s="68"/>
+      <c r="AL55" s="69"/>
+      <c r="AM55" s="69"/>
+      <c r="AN55" s="70"/>
       <c r="AO55" s="10"/>
       <c r="AP55" s="33"/>
       <c r="AQ55" s="33"/>
@@ -4764,14 +4775,14 @@
       <c r="AZ55" s="36"/>
     </row>
     <row r="56" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A56" s="64"/>
-      <c r="B56" s="66" t="s">
+      <c r="A56" s="97"/>
+      <c r="B56" s="77" t="s">
         <v>20</v>
       </c>
-      <c r="C56" s="61">
+      <c r="C56" s="78">
         <v>0.5</v>
       </c>
-      <c r="D56" s="61">
+      <c r="D56" s="78">
         <v>0</v>
       </c>
       <c r="E56" s="10"/>
@@ -4786,10 +4797,10 @@
       <c r="N56" s="11"/>
       <c r="O56" s="11"/>
       <c r="P56" s="12"/>
-      <c r="Q56" s="55"/>
-      <c r="R56" s="56"/>
-      <c r="S56" s="56"/>
-      <c r="T56" s="57"/>
+      <c r="Q56" s="68"/>
+      <c r="R56" s="69"/>
+      <c r="S56" s="69"/>
+      <c r="T56" s="70"/>
       <c r="U56" s="35"/>
       <c r="V56" s="33"/>
       <c r="W56" s="33"/>
@@ -4806,10 +4817,10 @@
       <c r="AH56" s="11"/>
       <c r="AI56" s="11"/>
       <c r="AJ56" s="36"/>
-      <c r="AK56" s="55"/>
-      <c r="AL56" s="56"/>
-      <c r="AM56" s="56"/>
-      <c r="AN56" s="57"/>
+      <c r="AK56" s="68"/>
+      <c r="AL56" s="69"/>
+      <c r="AM56" s="69"/>
+      <c r="AN56" s="70"/>
       <c r="AO56" s="10"/>
       <c r="AP56" s="11"/>
       <c r="AQ56" s="11"/>
@@ -4818,7 +4829,7 @@
       <c r="AT56" s="11"/>
       <c r="AU56" s="11"/>
       <c r="AV56" s="36"/>
-      <c r="AW56" s="106">
+      <c r="AW56" s="53">
         <v>0.5</v>
       </c>
       <c r="AX56" s="11"/>
@@ -4826,10 +4837,10 @@
       <c r="AZ56" s="36"/>
     </row>
     <row r="57" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A57" s="64"/>
-      <c r="B57" s="67"/>
-      <c r="C57" s="62"/>
-      <c r="D57" s="62"/>
+      <c r="A57" s="97"/>
+      <c r="B57" s="86"/>
+      <c r="C57" s="79"/>
+      <c r="D57" s="79"/>
       <c r="E57" s="10"/>
       <c r="F57" s="11"/>
       <c r="G57" s="11"/>
@@ -4842,10 +4853,10 @@
       <c r="N57" s="11"/>
       <c r="O57" s="11"/>
       <c r="P57" s="12"/>
-      <c r="Q57" s="55"/>
-      <c r="R57" s="56"/>
-      <c r="S57" s="56"/>
-      <c r="T57" s="57"/>
+      <c r="Q57" s="68"/>
+      <c r="R57" s="69"/>
+      <c r="S57" s="69"/>
+      <c r="T57" s="70"/>
       <c r="U57" s="35"/>
       <c r="V57" s="33"/>
       <c r="W57" s="33"/>
@@ -4862,10 +4873,10 @@
       <c r="AH57" s="11"/>
       <c r="AI57" s="11"/>
       <c r="AJ57" s="36"/>
-      <c r="AK57" s="55"/>
-      <c r="AL57" s="56"/>
-      <c r="AM57" s="56"/>
-      <c r="AN57" s="57"/>
+      <c r="AK57" s="68"/>
+      <c r="AL57" s="69"/>
+      <c r="AM57" s="69"/>
+      <c r="AN57" s="70"/>
       <c r="AO57" s="10"/>
       <c r="AP57" s="11"/>
       <c r="AQ57" s="11"/>
@@ -4880,14 +4891,14 @@
       <c r="AZ57" s="36"/>
     </row>
     <row r="58" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A58" s="64"/>
-      <c r="B58" s="72" t="s">
+      <c r="A58" s="97"/>
+      <c r="B58" s="75" t="s">
         <v>21</v>
       </c>
-      <c r="C58" s="62">
+      <c r="C58" s="79">
         <v>1.5</v>
       </c>
-      <c r="D58" s="71">
+      <c r="D58" s="83">
         <v>0</v>
       </c>
       <c r="E58" s="10"/>
@@ -4902,10 +4913,10 @@
       <c r="N58" s="11"/>
       <c r="O58" s="11"/>
       <c r="P58" s="12"/>
-      <c r="Q58" s="55"/>
-      <c r="R58" s="56"/>
-      <c r="S58" s="56"/>
-      <c r="T58" s="57"/>
+      <c r="Q58" s="68"/>
+      <c r="R58" s="69"/>
+      <c r="S58" s="69"/>
+      <c r="T58" s="70"/>
       <c r="U58" s="35"/>
       <c r="V58" s="33"/>
       <c r="W58" s="33"/>
@@ -4922,10 +4933,10 @@
       <c r="AH58" s="11"/>
       <c r="AI58" s="11"/>
       <c r="AJ58" s="36"/>
-      <c r="AK58" s="55"/>
-      <c r="AL58" s="56"/>
-      <c r="AM58" s="56"/>
-      <c r="AN58" s="57"/>
+      <c r="AK58" s="68"/>
+      <c r="AL58" s="69"/>
+      <c r="AM58" s="69"/>
+      <c r="AN58" s="70"/>
       <c r="AO58" s="35"/>
       <c r="AP58" s="33"/>
       <c r="AQ58" s="33"/>
@@ -4934,7 +4945,7 @@
       <c r="AT58" s="11"/>
       <c r="AU58" s="11"/>
       <c r="AV58" s="36"/>
-      <c r="AW58" s="106">
+      <c r="AW58" s="53">
         <v>1.5</v>
       </c>
       <c r="AX58" s="11"/>
@@ -4942,10 +4953,10 @@
       <c r="AZ58" s="36"/>
     </row>
     <row r="59" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="65"/>
-      <c r="B59" s="73"/>
-      <c r="C59" s="74"/>
-      <c r="D59" s="75"/>
+      <c r="A59" s="98"/>
+      <c r="B59" s="100"/>
+      <c r="C59" s="91"/>
+      <c r="D59" s="92"/>
       <c r="E59" s="16"/>
       <c r="F59" s="17"/>
       <c r="G59" s="17"/>
@@ -4958,10 +4969,10 @@
       <c r="N59" s="17"/>
       <c r="O59" s="17"/>
       <c r="P59" s="18"/>
-      <c r="Q59" s="55"/>
-      <c r="R59" s="56"/>
-      <c r="S59" s="56"/>
-      <c r="T59" s="57"/>
+      <c r="Q59" s="68"/>
+      <c r="R59" s="69"/>
+      <c r="S59" s="69"/>
+      <c r="T59" s="70"/>
       <c r="U59" s="34"/>
       <c r="V59" s="38"/>
       <c r="W59" s="38"/>
@@ -4978,10 +4989,10 @@
       <c r="AH59" s="17"/>
       <c r="AI59" s="17"/>
       <c r="AJ59" s="18"/>
-      <c r="AK59" s="55"/>
-      <c r="AL59" s="56"/>
-      <c r="AM59" s="56"/>
-      <c r="AN59" s="57"/>
+      <c r="AK59" s="68"/>
+      <c r="AL59" s="69"/>
+      <c r="AM59" s="69"/>
+      <c r="AN59" s="70"/>
       <c r="AO59" s="34"/>
       <c r="AP59" s="38"/>
       <c r="AQ59" s="38"/>
@@ -4996,16 +5007,16 @@
       <c r="AZ59" s="18"/>
     </row>
     <row r="60" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A60" s="63" t="s">
+      <c r="A60" s="96" t="s">
         <v>14</v>
       </c>
-      <c r="B60" s="66" t="s">
+      <c r="B60" s="77" t="s">
         <v>23</v>
       </c>
-      <c r="C60" s="61">
+      <c r="C60" s="78">
         <v>6</v>
       </c>
-      <c r="D60" s="61">
+      <c r="D60" s="78">
         <v>0</v>
       </c>
       <c r="E60" s="10"/>
@@ -5020,10 +5031,10 @@
       <c r="N60" s="11"/>
       <c r="O60" s="11"/>
       <c r="P60" s="12"/>
-      <c r="Q60" s="55"/>
-      <c r="R60" s="56"/>
-      <c r="S60" s="56"/>
-      <c r="T60" s="57"/>
+      <c r="Q60" s="68"/>
+      <c r="R60" s="69"/>
+      <c r="S60" s="69"/>
+      <c r="T60" s="70"/>
       <c r="U60" s="35"/>
       <c r="V60" s="33"/>
       <c r="W60" s="33"/>
@@ -5040,10 +5051,10 @@
       <c r="AH60" s="11"/>
       <c r="AI60" s="11"/>
       <c r="AJ60" s="12"/>
-      <c r="AK60" s="55"/>
-      <c r="AL60" s="56"/>
-      <c r="AM60" s="56"/>
-      <c r="AN60" s="57"/>
+      <c r="AK60" s="68"/>
+      <c r="AL60" s="69"/>
+      <c r="AM60" s="69"/>
+      <c r="AN60" s="70"/>
       <c r="AO60" s="35"/>
       <c r="AP60" s="33"/>
       <c r="AQ60" s="33"/>
@@ -5052,16 +5063,16 @@
       <c r="AT60" s="11"/>
       <c r="AU60" s="11"/>
       <c r="AV60" s="12"/>
-      <c r="AW60" s="110"/>
-      <c r="AX60" s="104"/>
-      <c r="AY60" s="104"/>
-      <c r="AZ60" s="105"/>
+      <c r="AW60" s="57"/>
+      <c r="AX60" s="51"/>
+      <c r="AY60" s="51"/>
+      <c r="AZ60" s="52"/>
     </row>
     <row r="61" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="64"/>
-      <c r="B61" s="67"/>
-      <c r="C61" s="62"/>
-      <c r="D61" s="62"/>
+      <c r="A61" s="97"/>
+      <c r="B61" s="86"/>
+      <c r="C61" s="79"/>
+      <c r="D61" s="79"/>
       <c r="E61" s="10"/>
       <c r="F61" s="11"/>
       <c r="G61" s="11"/>
@@ -5074,10 +5085,10 @@
       <c r="N61" s="11"/>
       <c r="O61" s="11"/>
       <c r="P61" s="12"/>
-      <c r="Q61" s="55"/>
-      <c r="R61" s="56"/>
-      <c r="S61" s="56"/>
-      <c r="T61" s="57"/>
+      <c r="Q61" s="68"/>
+      <c r="R61" s="69"/>
+      <c r="S61" s="69"/>
+      <c r="T61" s="70"/>
       <c r="U61" s="35"/>
       <c r="V61" s="33"/>
       <c r="W61" s="33"/>
@@ -5094,10 +5105,10 @@
       <c r="AH61" s="11"/>
       <c r="AI61" s="11"/>
       <c r="AJ61" s="12"/>
-      <c r="AK61" s="55"/>
-      <c r="AL61" s="56"/>
-      <c r="AM61" s="56"/>
-      <c r="AN61" s="57"/>
+      <c r="AK61" s="68"/>
+      <c r="AL61" s="69"/>
+      <c r="AM61" s="69"/>
+      <c r="AN61" s="70"/>
       <c r="AO61" s="10"/>
       <c r="AP61" s="11"/>
       <c r="AQ61" s="11"/>
@@ -5112,14 +5123,14 @@
       <c r="AZ61" s="36"/>
     </row>
     <row r="62" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="64"/>
-      <c r="B62" s="66" t="s">
+      <c r="A62" s="97"/>
+      <c r="B62" s="77" t="s">
         <v>6</v>
       </c>
-      <c r="C62" s="61">
+      <c r="C62" s="78">
         <v>0</v>
       </c>
-      <c r="D62" s="61">
+      <c r="D62" s="78">
         <v>0</v>
       </c>
       <c r="E62" s="10"/>
@@ -5134,10 +5145,10 @@
       <c r="N62" s="11"/>
       <c r="O62" s="11"/>
       <c r="P62" s="12"/>
-      <c r="Q62" s="55"/>
-      <c r="R62" s="56"/>
-      <c r="S62" s="56"/>
-      <c r="T62" s="57"/>
+      <c r="Q62" s="68"/>
+      <c r="R62" s="69"/>
+      <c r="S62" s="69"/>
+      <c r="T62" s="70"/>
       <c r="U62" s="35"/>
       <c r="V62" s="33"/>
       <c r="W62" s="33"/>
@@ -5154,10 +5165,10 @@
       <c r="AH62" s="11"/>
       <c r="AI62" s="11"/>
       <c r="AJ62" s="12"/>
-      <c r="AK62" s="55"/>
-      <c r="AL62" s="56"/>
-      <c r="AM62" s="56"/>
-      <c r="AN62" s="57"/>
+      <c r="AK62" s="68"/>
+      <c r="AL62" s="69"/>
+      <c r="AM62" s="69"/>
+      <c r="AN62" s="70"/>
       <c r="AO62" s="10"/>
       <c r="AP62" s="11"/>
       <c r="AQ62" s="11"/>
@@ -5172,10 +5183,10 @@
       <c r="AZ62" s="12"/>
     </row>
     <row r="63" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="65"/>
-      <c r="B63" s="68"/>
-      <c r="C63" s="62"/>
-      <c r="D63" s="62"/>
+      <c r="A63" s="98"/>
+      <c r="B63" s="102"/>
+      <c r="C63" s="79"/>
+      <c r="D63" s="79"/>
       <c r="E63" s="16"/>
       <c r="F63" s="17"/>
       <c r="G63" s="17"/>
@@ -5188,10 +5199,10 @@
       <c r="N63" s="17"/>
       <c r="O63" s="17"/>
       <c r="P63" s="18"/>
-      <c r="Q63" s="58"/>
-      <c r="R63" s="59"/>
-      <c r="S63" s="59"/>
-      <c r="T63" s="60"/>
+      <c r="Q63" s="71"/>
+      <c r="R63" s="72"/>
+      <c r="S63" s="72"/>
+      <c r="T63" s="73"/>
       <c r="U63" s="16"/>
       <c r="V63" s="17"/>
       <c r="W63" s="17"/>
@@ -5208,10 +5219,10 @@
       <c r="AH63" s="17"/>
       <c r="AI63" s="17"/>
       <c r="AJ63" s="18"/>
-      <c r="AK63" s="58"/>
-      <c r="AL63" s="59"/>
-      <c r="AM63" s="59"/>
-      <c r="AN63" s="60"/>
+      <c r="AK63" s="71"/>
+      <c r="AL63" s="72"/>
+      <c r="AM63" s="72"/>
+      <c r="AN63" s="73"/>
       <c r="AO63" s="16"/>
       <c r="AP63" s="17"/>
       <c r="AQ63" s="17"/>
@@ -5235,7 +5246,7 @@
       </c>
       <c r="D64" s="5">
         <f>SUM(D4:D63)</f>
-        <v>20</v>
+        <v>9.5</v>
       </c>
       <c r="AQ64" s="6"/>
       <c r="AR64" s="6"/>
@@ -5243,6 +5254,107 @@
     <row r="65" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="125">
+    <mergeCell ref="A28:A53"/>
+    <mergeCell ref="A54:A59"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="A60:A63"/>
+    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="A6:A11"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="A12:A25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="AK1:AN1"/>
+    <mergeCell ref="AO2:AR2"/>
+    <mergeCell ref="AO1:AR1"/>
+    <mergeCell ref="AG2:AJ2"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="AS1:AV1"/>
+    <mergeCell ref="AS2:AV2"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="AC1:AF1"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="U2:X2"/>
+    <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="M1:P1"/>
+    <mergeCell ref="Q1:T1"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="AG1:AJ1"/>
     <mergeCell ref="AW1:AZ1"/>
     <mergeCell ref="AW2:AZ2"/>
     <mergeCell ref="Q6:T63"/>
@@ -5267,107 +5379,6 @@
     <mergeCell ref="B34:B35"/>
     <mergeCell ref="C34:C35"/>
     <mergeCell ref="B38:B39"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="AS1:AV1"/>
-    <mergeCell ref="AS2:AV2"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="M2:P2"/>
-    <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="U2:X2"/>
-    <mergeCell ref="Y2:AB2"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E1:H1"/>
-    <mergeCell ref="I1:L1"/>
-    <mergeCell ref="M1:P1"/>
-    <mergeCell ref="Q1:T1"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AK1:AN1"/>
-    <mergeCell ref="AO2:AR2"/>
-    <mergeCell ref="AO1:AR1"/>
-    <mergeCell ref="AG2:AJ2"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="A6:A11"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="A12:A25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="A60:A63"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="D62:D63"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="A28:A53"/>
-    <mergeCell ref="A54:A59"/>
-    <mergeCell ref="A26:A27"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>